<commit_message>
feat: implement OBE curriculum documentation and management tools for SISTEKIN 2026
</commit_message>
<xml_diff>
--- a/KURIKULUM2026_REVISI/011_IMPLEMENTASI_OBE_SISTEKIN2026_TABLES.xlsx
+++ b/KURIKULUM2026_REVISI/011_IMPLEMENTASI_OBE_SISTEKIN2026_TABLES.xlsx
@@ -592,11 +592,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="80" customWidth="1" min="2" max="2"/>
+    <col width="85" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
@@ -659,7 +659,7 @@
       <c r="A9" s="10" t="inlineStr"/>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>Catatan Data Final:</t>
+          <t>Parameter Kurikulum Final Terverifikasi:</t>
         </is>
       </c>
     </row>
@@ -695,19 +695,11 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="19.8" customHeight="1">
-      <c r="A14" s="10" t="inlineStr"/>
-      <c r="B14" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ✓  STI-405 Dasar Keamanan Informasi = 2 SKS (Teori)</t>
-        </is>
-      </c>
-    </row>
     <row r="15" ht="19.8" customHeight="1">
       <c r="A15" s="10" t="inlineStr"/>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ✓  STI-602 Smart City &amp; Pemerintahan Digital = 2 SKS (Teori)</t>
+          <t xml:space="preserve">  ✓  STI-405 Dasar Keamanan Informasi = 2 SKS &amp; STI-602 Smart City = 2 SKS</t>
         </is>
       </c>
     </row>
@@ -715,7 +707,15 @@
       <c r="A16" s="10" t="inlineStr"/>
       <c r="B16" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ✓  MKU-401A Agama II &amp; MKU-402 Kewirausahaan II = 0 SKS (Kebijakan UWG)</t>
+          <t xml:space="preserve">  ✓  MKU-406 Agama II &amp; MKU-508 Kewirausahaan II = 0 SKS (Kebijakan UWG)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="19.8" customHeight="1">
+      <c r="A17" s="10" t="inlineStr"/>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ✓  Skema 4x Asesmen Baku per MK (Tugas 1 [20%], UTS [25-30%], Tugas 2 [20-25%], UAS [30%])</t>
         </is>
       </c>
     </row>
@@ -748,14 +748,14 @@
     <col width="11.5" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="13" t="inlineStr">
         <is>
           <t>SISTEKIN 2026 — Sheet 9: Template Evaluasi OBE - STI-601 (Integrasi AI)</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1">
+    <row r="2" ht="16" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
           <t>TEMPLATE EVALUASI OBE - STI-601 Integrasi Layanan Cerdas Berbasis AI</t>
@@ -824,7 +824,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1">
+    <row r="4" ht="16" customHeight="1">
       <c r="A4" s="16" t="inlineStr">
         <is>
           <t>1</t>
@@ -842,7 +842,7 @@
       <c r="K4" s="18" t="inlineStr"/>
       <c r="L4" s="18" t="inlineStr"/>
     </row>
-    <row r="5" ht="15" customHeight="1">
+    <row r="5" ht="16" customHeight="1">
       <c r="A5" s="17" t="inlineStr">
         <is>
           <t>2</t>
@@ -860,7 +860,7 @@
       <c r="K5" s="19" t="inlineStr"/>
       <c r="L5" s="19" t="inlineStr"/>
     </row>
-    <row r="6" ht="15" customHeight="1">
+    <row r="6" ht="16" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
           <t>3</t>
@@ -878,7 +878,7 @@
       <c r="K6" s="18" t="inlineStr"/>
       <c r="L6" s="18" t="inlineStr"/>
     </row>
-    <row r="7" ht="15" customHeight="1">
+    <row r="7" ht="16" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
           <t>4</t>
@@ -896,7 +896,7 @@
       <c r="K7" s="19" t="inlineStr"/>
       <c r="L7" s="19" t="inlineStr"/>
     </row>
-    <row r="8" ht="15" customHeight="1">
+    <row r="8" ht="16" customHeight="1">
       <c r="A8" s="16" t="inlineStr">
         <is>
           <t>5</t>
@@ -914,7 +914,7 @@
       <c r="K8" s="18" t="inlineStr"/>
       <c r="L8" s="18" t="inlineStr"/>
     </row>
-    <row r="9" ht="15" customHeight="1">
+    <row r="9" ht="16" customHeight="1">
       <c r="A9" s="17" t="inlineStr">
         <is>
           <t>10</t>
@@ -932,7 +932,7 @@
       <c r="K9" s="19" t="inlineStr"/>
       <c r="L9" s="19" t="inlineStr"/>
     </row>
-    <row r="10" ht="15" customHeight="1">
+    <row r="10" ht="16" customHeight="1">
       <c r="A10" s="16" t="inlineStr">
         <is>
           <t>15</t>
@@ -950,7 +950,7 @@
       <c r="K10" s="18" t="inlineStr"/>
       <c r="L10" s="18" t="inlineStr"/>
     </row>
-    <row r="11" ht="15" customHeight="1">
+    <row r="11" ht="16" customHeight="1">
       <c r="A11" s="17" t="inlineStr">
         <is>
           <t>20</t>
@@ -968,7 +968,7 @@
       <c r="K11" s="19" t="inlineStr"/>
       <c r="L11" s="19" t="inlineStr"/>
     </row>
-    <row r="12" ht="15" customHeight="1">
+    <row r="12" ht="16" customHeight="1">
       <c r="A12" s="16" t="inlineStr">
         <is>
           <t>25</t>
@@ -986,7 +986,7 @@
       <c r="K12" s="18" t="inlineStr"/>
       <c r="L12" s="18" t="inlineStr"/>
     </row>
-    <row r="13" ht="15" customHeight="1">
+    <row r="13" ht="16" customHeight="1">
       <c r="A13" s="17" t="inlineStr">
         <is>
           <t>30</t>
@@ -1004,7 +1004,7 @@
       <c r="K13" s="19" t="inlineStr"/>
       <c r="L13" s="19" t="inlineStr"/>
     </row>
-    <row r="14" ht="15" customHeight="1">
+    <row r="14" ht="16" customHeight="1">
       <c r="A14" s="20" t="inlineStr">
         <is>
           <t>Ringkasan Kelas</t>
@@ -1034,7 +1034,7 @@
       <c r="K14" s="20" t="inlineStr"/>
       <c r="L14" s="20" t="inlineStr"/>
     </row>
-    <row r="15" ht="15" customHeight="1">
+    <row r="15" ht="16" customHeight="1">
       <c r="A15" s="20" t="inlineStr">
         <is>
           <t>% Mahasiswa &gt;= 75</t>
@@ -1090,14 +1090,14 @@
     <col width="11.5" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="13" t="inlineStr">
         <is>
           <t>SISTEKIN 2026 — Sheet 10: Template Evaluasi OBE - STI-401 (Machine Learning)</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1">
+    <row r="2" ht="16" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
           <t>TEMPLATE EVALUASI OBE - STI-401 Machine Learning (+P)</t>
@@ -1171,7 +1171,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1">
+    <row r="4" ht="16" customHeight="1">
       <c r="A4" s="16" t="inlineStr">
         <is>
           <t>1</t>
@@ -1190,7 +1190,7 @@
       <c r="L4" s="18" t="inlineStr"/>
       <c r="M4" s="18" t="inlineStr"/>
     </row>
-    <row r="5" ht="15" customHeight="1">
+    <row r="5" ht="16" customHeight="1">
       <c r="A5" s="17" t="inlineStr">
         <is>
           <t>2</t>
@@ -1209,7 +1209,7 @@
       <c r="L5" s="19" t="inlineStr"/>
       <c r="M5" s="19" t="inlineStr"/>
     </row>
-    <row r="6" ht="15" customHeight="1">
+    <row r="6" ht="16" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
           <t>3</t>
@@ -1228,7 +1228,7 @@
       <c r="L6" s="18" t="inlineStr"/>
       <c r="M6" s="18" t="inlineStr"/>
     </row>
-    <row r="7" ht="15" customHeight="1">
+    <row r="7" ht="16" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
           <t>4</t>
@@ -1247,7 +1247,7 @@
       <c r="L7" s="19" t="inlineStr"/>
       <c r="M7" s="19" t="inlineStr"/>
     </row>
-    <row r="8" ht="15" customHeight="1">
+    <row r="8" ht="16" customHeight="1">
       <c r="A8" s="16" t="inlineStr">
         <is>
           <t>5</t>
@@ -1266,7 +1266,7 @@
       <c r="L8" s="18" t="inlineStr"/>
       <c r="M8" s="18" t="inlineStr"/>
     </row>
-    <row r="9" ht="15" customHeight="1">
+    <row r="9" ht="16" customHeight="1">
       <c r="A9" s="17" t="inlineStr">
         <is>
           <t>10</t>
@@ -1285,7 +1285,7 @@
       <c r="L9" s="19" t="inlineStr"/>
       <c r="M9" s="19" t="inlineStr"/>
     </row>
-    <row r="10" ht="15" customHeight="1">
+    <row r="10" ht="16" customHeight="1">
       <c r="A10" s="16" t="inlineStr">
         <is>
           <t>15</t>
@@ -1304,7 +1304,7 @@
       <c r="L10" s="18" t="inlineStr"/>
       <c r="M10" s="18" t="inlineStr"/>
     </row>
-    <row r="11" ht="15" customHeight="1">
+    <row r="11" ht="16" customHeight="1">
       <c r="A11" s="17" t="inlineStr">
         <is>
           <t>20</t>
@@ -1323,7 +1323,7 @@
       <c r="L11" s="19" t="inlineStr"/>
       <c r="M11" s="19" t="inlineStr"/>
     </row>
-    <row r="12" ht="15" customHeight="1">
+    <row r="12" ht="16" customHeight="1">
       <c r="A12" s="16" t="inlineStr">
         <is>
           <t>25</t>
@@ -1342,7 +1342,7 @@
       <c r="L12" s="18" t="inlineStr"/>
       <c r="M12" s="18" t="inlineStr"/>
     </row>
-    <row r="13" ht="15" customHeight="1">
+    <row r="13" ht="16" customHeight="1">
       <c r="A13" s="17" t="inlineStr">
         <is>
           <t>30</t>
@@ -1361,7 +1361,7 @@
       <c r="L13" s="19" t="inlineStr"/>
       <c r="M13" s="19" t="inlineStr"/>
     </row>
-    <row r="14" ht="15" customHeight="1">
+    <row r="14" ht="16" customHeight="1">
       <c r="A14" s="20" t="inlineStr">
         <is>
           <t>Ringkasan Kelas</t>
@@ -1392,7 +1392,7 @@
       <c r="L14" s="20" t="inlineStr"/>
       <c r="M14" s="20" t="inlineStr"/>
     </row>
-    <row r="15" ht="15" customHeight="1">
+    <row r="15" ht="16" customHeight="1">
       <c r="A15" s="20" t="inlineStr">
         <is>
           <t>% Mahasiswa &gt;= 75</t>
@@ -1448,14 +1448,14 @@
     <col width="11.5" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="13" t="inlineStr">
         <is>
           <t>SISTEKIN 2026 — Sheet 11: Template Evaluasi OBE - STI-303 (UI/UX)</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1">
+    <row r="2" ht="16" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
           <t>TEMPLATE EVALUASI OBE - STI-303 UI/UX Design &amp; Prototyping (+P)</t>
@@ -1524,7 +1524,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1">
+    <row r="4" ht="16" customHeight="1">
       <c r="A4" s="16" t="inlineStr">
         <is>
           <t>1</t>
@@ -1542,7 +1542,7 @@
       <c r="K4" s="18" t="inlineStr"/>
       <c r="L4" s="18" t="inlineStr"/>
     </row>
-    <row r="5" ht="15" customHeight="1">
+    <row r="5" ht="16" customHeight="1">
       <c r="A5" s="17" t="inlineStr">
         <is>
           <t>2</t>
@@ -1560,7 +1560,7 @@
       <c r="K5" s="19" t="inlineStr"/>
       <c r="L5" s="19" t="inlineStr"/>
     </row>
-    <row r="6" ht="15" customHeight="1">
+    <row r="6" ht="16" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
           <t>3</t>
@@ -1578,7 +1578,7 @@
       <c r="K6" s="18" t="inlineStr"/>
       <c r="L6" s="18" t="inlineStr"/>
     </row>
-    <row r="7" ht="15" customHeight="1">
+    <row r="7" ht="16" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
           <t>4</t>
@@ -1596,7 +1596,7 @@
       <c r="K7" s="19" t="inlineStr"/>
       <c r="L7" s="19" t="inlineStr"/>
     </row>
-    <row r="8" ht="15" customHeight="1">
+    <row r="8" ht="16" customHeight="1">
       <c r="A8" s="16" t="inlineStr">
         <is>
           <t>5</t>
@@ -1614,7 +1614,7 @@
       <c r="K8" s="18" t="inlineStr"/>
       <c r="L8" s="18" t="inlineStr"/>
     </row>
-    <row r="9" ht="15" customHeight="1">
+    <row r="9" ht="16" customHeight="1">
       <c r="A9" s="17" t="inlineStr">
         <is>
           <t>10</t>
@@ -1632,7 +1632,7 @@
       <c r="K9" s="19" t="inlineStr"/>
       <c r="L9" s="19" t="inlineStr"/>
     </row>
-    <row r="10" ht="15" customHeight="1">
+    <row r="10" ht="16" customHeight="1">
       <c r="A10" s="16" t="inlineStr">
         <is>
           <t>15</t>
@@ -1650,7 +1650,7 @@
       <c r="K10" s="18" t="inlineStr"/>
       <c r="L10" s="18" t="inlineStr"/>
     </row>
-    <row r="11" ht="15" customHeight="1">
+    <row r="11" ht="16" customHeight="1">
       <c r="A11" s="17" t="inlineStr">
         <is>
           <t>20</t>
@@ -1668,7 +1668,7 @@
       <c r="K11" s="19" t="inlineStr"/>
       <c r="L11" s="19" t="inlineStr"/>
     </row>
-    <row r="12" ht="15" customHeight="1">
+    <row r="12" ht="16" customHeight="1">
       <c r="A12" s="16" t="inlineStr">
         <is>
           <t>25</t>
@@ -1686,7 +1686,7 @@
       <c r="K12" s="18" t="inlineStr"/>
       <c r="L12" s="18" t="inlineStr"/>
     </row>
-    <row r="13" ht="15" customHeight="1">
+    <row r="13" ht="16" customHeight="1">
       <c r="A13" s="17" t="inlineStr">
         <is>
           <t>30</t>
@@ -1704,7 +1704,7 @@
       <c r="K13" s="19" t="inlineStr"/>
       <c r="L13" s="19" t="inlineStr"/>
     </row>
-    <row r="14" ht="15" customHeight="1">
+    <row r="14" ht="16" customHeight="1">
       <c r="A14" s="20" t="inlineStr">
         <is>
           <t>Ringkasan Kelas</t>
@@ -1734,7 +1734,7 @@
       <c r="K14" s="20" t="inlineStr"/>
       <c r="L14" s="20" t="inlineStr"/>
     </row>
-    <row r="15" ht="15" customHeight="1">
+    <row r="15" ht="16" customHeight="1">
       <c r="A15" s="20" t="inlineStr">
         <is>
           <t>% Mahasiswa &gt;= 75</t>
@@ -1789,14 +1789,14 @@
     <col width="11.5" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="13" t="inlineStr">
         <is>
           <t>SISTEKIN 2026 — Sheet 12: Template Evaluasi OBE - STI-603 (Keamanan)</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1">
+    <row r="2" ht="16" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
           <t>TEMPLATE EVALUASI OBE - STI-603 Keamanan Informasi Lanjut</t>
@@ -1865,7 +1865,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1">
+    <row r="4" ht="16" customHeight="1">
       <c r="A4" s="16" t="inlineStr">
         <is>
           <t>1</t>
@@ -1883,7 +1883,7 @@
       <c r="K4" s="18" t="inlineStr"/>
       <c r="L4" s="18" t="inlineStr"/>
     </row>
-    <row r="5" ht="15" customHeight="1">
+    <row r="5" ht="16" customHeight="1">
       <c r="A5" s="17" t="inlineStr">
         <is>
           <t>2</t>
@@ -1901,7 +1901,7 @@
       <c r="K5" s="19" t="inlineStr"/>
       <c r="L5" s="19" t="inlineStr"/>
     </row>
-    <row r="6" ht="15" customHeight="1">
+    <row r="6" ht="16" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
           <t>3</t>
@@ -1919,7 +1919,7 @@
       <c r="K6" s="18" t="inlineStr"/>
       <c r="L6" s="18" t="inlineStr"/>
     </row>
-    <row r="7" ht="15" customHeight="1">
+    <row r="7" ht="16" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
           <t>4</t>
@@ -1937,7 +1937,7 @@
       <c r="K7" s="19" t="inlineStr"/>
       <c r="L7" s="19" t="inlineStr"/>
     </row>
-    <row r="8" ht="15" customHeight="1">
+    <row r="8" ht="16" customHeight="1">
       <c r="A8" s="16" t="inlineStr">
         <is>
           <t>5</t>
@@ -1955,7 +1955,7 @@
       <c r="K8" s="18" t="inlineStr"/>
       <c r="L8" s="18" t="inlineStr"/>
     </row>
-    <row r="9" ht="15" customHeight="1">
+    <row r="9" ht="16" customHeight="1">
       <c r="A9" s="17" t="inlineStr">
         <is>
           <t>10</t>
@@ -1973,7 +1973,7 @@
       <c r="K9" s="19" t="inlineStr"/>
       <c r="L9" s="19" t="inlineStr"/>
     </row>
-    <row r="10" ht="15" customHeight="1">
+    <row r="10" ht="16" customHeight="1">
       <c r="A10" s="16" t="inlineStr">
         <is>
           <t>15</t>
@@ -1991,7 +1991,7 @@
       <c r="K10" s="18" t="inlineStr"/>
       <c r="L10" s="18" t="inlineStr"/>
     </row>
-    <row r="11" ht="15" customHeight="1">
+    <row r="11" ht="16" customHeight="1">
       <c r="A11" s="17" t="inlineStr">
         <is>
           <t>20</t>
@@ -2009,7 +2009,7 @@
       <c r="K11" s="19" t="inlineStr"/>
       <c r="L11" s="19" t="inlineStr"/>
     </row>
-    <row r="12" ht="15" customHeight="1">
+    <row r="12" ht="16" customHeight="1">
       <c r="A12" s="16" t="inlineStr">
         <is>
           <t>25</t>
@@ -2027,7 +2027,7 @@
       <c r="K12" s="18" t="inlineStr"/>
       <c r="L12" s="18" t="inlineStr"/>
     </row>
-    <row r="13" ht="15" customHeight="1">
+    <row r="13" ht="16" customHeight="1">
       <c r="A13" s="17" t="inlineStr">
         <is>
           <t>30</t>
@@ -2045,7 +2045,7 @@
       <c r="K13" s="19" t="inlineStr"/>
       <c r="L13" s="19" t="inlineStr"/>
     </row>
-    <row r="14" ht="15" customHeight="1">
+    <row r="14" ht="16" customHeight="1">
       <c r="A14" s="20" t="inlineStr">
         <is>
           <t>Ringkasan Kelas</t>
@@ -2075,7 +2075,7 @@
       <c r="K14" s="20" t="inlineStr"/>
       <c r="L14" s="20" t="inlineStr"/>
     </row>
-    <row r="15" ht="15" customHeight="1">
+    <row r="15" ht="16" customHeight="1">
       <c r="A15" s="20" t="inlineStr">
         <is>
           <t>% Mahasiswa &gt;= 75</t>
@@ -2125,14 +2125,14 @@
     <col width="16.1" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="13" t="inlineStr">
         <is>
           <t>SISTEKIN 2026 — Sheet 13: Rekapitulasi Ketercapaian CPL Program Studi</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1">
+    <row r="2" ht="16" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
           <t>TEMPLATE REKAPITULASI KETERCAPAIAN CPL PROGRAM STUDI SISTEKIN 2026 (Dok. 008)</t>
@@ -2176,7 +2176,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1">
+    <row r="4" ht="16" customHeight="1">
       <c r="A4" s="16" t="inlineStr">
         <is>
           <t>S1</t>
@@ -2194,7 +2194,7 @@
       </c>
       <c r="D4" s="16" t="inlineStr">
         <is>
-          <t>FST-610 Capstone, FST-612 PKL, MKU-203 KPM, FST-714 Skripsi</t>
+          <t>FST-610 Capstone, FST-612 PKL, MKU-507 KPM, FST-714 Skripsi</t>
         </is>
       </c>
       <c r="E4" s="16" t="inlineStr">
@@ -2209,7 +2209,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1">
+    <row r="5" ht="16" customHeight="1">
       <c r="A5" s="17" t="inlineStr">
         <is>
           <t>KU1</t>
@@ -2242,7 +2242,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1">
+    <row r="6" ht="16" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
           <t>KU2</t>
@@ -2260,7 +2260,7 @@
       </c>
       <c r="D6" s="16" t="inlineStr">
         <is>
-          <t>FST-610 Capstone, FST-611 Metpen, MKU-203 KPM, FST-714 Skripsi</t>
+          <t>FST-610 Capstone, FST-611 Metpen, MKU-507 KPM, FST-714 Skripsi</t>
         </is>
       </c>
       <c r="E6" s="16" t="inlineStr">
@@ -2275,7 +2275,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1">
+    <row r="7" ht="16" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
           <t>KU3</t>
@@ -2308,7 +2308,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1">
+    <row r="8" ht="16" customHeight="1">
       <c r="A8" s="16" t="inlineStr">
         <is>
           <t>P1</t>
@@ -2341,7 +2341,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1">
+    <row r="9" ht="16" customHeight="1">
       <c r="A9" s="17" t="inlineStr">
         <is>
           <t>P2</t>
@@ -2374,7 +2374,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1">
+    <row r="10" ht="16" customHeight="1">
       <c r="A10" s="16" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2407,7 +2407,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1">
+    <row r="11" ht="16" customHeight="1">
       <c r="A11" s="17" t="inlineStr">
         <is>
           <t>P4</t>
@@ -2440,7 +2440,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1">
+    <row r="12" ht="16" customHeight="1">
       <c r="A12" s="16" t="inlineStr">
         <is>
           <t>KK1</t>
@@ -2473,7 +2473,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1">
+    <row r="13" ht="16" customHeight="1">
       <c r="A13" s="17" t="inlineStr">
         <is>
           <t>KK2</t>
@@ -2506,7 +2506,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1">
+    <row r="14" ht="16" customHeight="1">
       <c r="A14" s="16" t="inlineStr">
         <is>
           <t>KK3</t>
@@ -2539,7 +2539,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="15" customHeight="1">
+    <row r="15" ht="16" customHeight="1">
       <c r="A15" s="17" t="inlineStr">
         <is>
           <t>KK4</t>
@@ -2572,7 +2572,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1">
+    <row r="16" ht="16" customHeight="1">
       <c r="A16" s="16" t="inlineStr">
         <is>
           <t>KK5</t>
@@ -2605,7 +2605,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="15" customHeight="1">
+    <row r="17" ht="16" customHeight="1">
       <c r="A17" s="17" t="inlineStr">
         <is>
           <t>KK6</t>
@@ -2665,14 +2665,14 @@
     <col width="16.1" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="13" t="inlineStr">
         <is>
           <t>SISTEKIN 2026 — Sheet 14: Ringkasan Implementasi OBE</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1">
+    <row r="2" ht="16" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
           <t>RINGKASAN IMPLEMENTASI MODUL OBE - S1 SISTEM DAN TEKNOLOGI INFORMASI 2026</t>
@@ -2707,7 +2707,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1">
+    <row r="4" ht="16" customHeight="1">
       <c r="A4" s="16" t="inlineStr">
         <is>
           <t>Profil Lulusan (PL)</t>
@@ -2735,7 +2735,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1">
+    <row r="5" ht="16" customHeight="1">
       <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Program Educational Objectives (PEO)</t>
@@ -2763,7 +2763,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1">
+    <row r="6" ht="16" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
           <t>CPL (Capaian Pembelajaran Lulusan)</t>
@@ -2791,7 +2791,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1">
+    <row r="7" ht="16" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
           <t>MK Wajib (Paket Ditempuh)</t>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1">
+    <row r="8" ht="16" customHeight="1">
       <c r="A8" s="16" t="inlineStr">
         <is>
           <t>MK Elektif Ditempuh (1 dari 3 Peminatan)</t>
@@ -2847,7 +2847,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1">
+    <row r="9" ht="16" customHeight="1">
       <c r="A9" s="20" t="inlineStr">
         <is>
           <t>Total MK Paket Ditempuh</t>
@@ -2875,7 +2875,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1">
+    <row r="10" ht="16" customHeight="1">
       <c r="A10" s="20" t="inlineStr">
         <is>
           <t>Total SKS Paket Ditempuh (Syarat Lulus)</t>
@@ -2903,7 +2903,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1">
+    <row r="11" ht="16" customHeight="1">
       <c r="A11" s="20" t="inlineStr">
         <is>
           <t>Total MK Portofolio Ditawarkan</t>
@@ -2931,7 +2931,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1">
+    <row r="12" ht="16" customHeight="1">
       <c r="A12" s="20" t="inlineStr">
         <is>
           <t>Total SKS Portofolio Ditawarkan</t>
@@ -2959,7 +2959,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1">
+    <row r="13" ht="16" customHeight="1">
       <c r="A13" s="17" t="inlineStr">
         <is>
           <t>Peminatan Spesialisasi</t>
@@ -2987,7 +2987,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1">
+    <row r="14" ht="16" customHeight="1">
       <c r="A14" s="16" t="inlineStr">
         <is>
           <t>Semester</t>
@@ -3015,7 +3015,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="15" customHeight="1">
+    <row r="15" ht="16" customHeight="1">
       <c r="A15" s="17" t="inlineStr">
         <is>
           <t>Syarat Lulus Minimal (Permendikbud 53/2023)</t>
@@ -3056,7 +3056,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1">
+    <row r="18" ht="16" customHeight="1">
       <c r="A18" s="16" t="inlineStr">
         <is>
           <t>1</t>
@@ -3068,7 +3068,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1">
+    <row r="19" ht="16" customHeight="1">
       <c r="A19" s="17" t="inlineStr">
         <is>
           <t>2</t>
@@ -3080,7 +3080,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="15" customHeight="1">
+    <row r="20" ht="16" customHeight="1">
       <c r="A20" s="16" t="inlineStr">
         <is>
           <t>3</t>
@@ -3092,7 +3092,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1">
+    <row r="21" ht="16" customHeight="1">
       <c r="A21" s="17" t="inlineStr">
         <is>
           <t>4</t>
@@ -3104,7 +3104,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="15" customHeight="1">
+    <row r="22" ht="16" customHeight="1">
       <c r="A22" s="16" t="inlineStr">
         <is>
           <t>5</t>
@@ -3116,7 +3116,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1">
+    <row r="23" ht="16" customHeight="1">
       <c r="A23" s="17" t="inlineStr">
         <is>
           <t>6</t>
@@ -3128,7 +3128,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="15" customHeight="1">
+    <row r="24" ht="16" customHeight="1">
       <c r="A24" s="16" t="inlineStr">
         <is>
           <t>7</t>
@@ -3136,7 +3136,7 @@
       </c>
       <c r="B24" s="16" t="inlineStr">
         <is>
-          <t>MKU-401A (Agama II) dan MKU-402 (Kewirausahaan II) = 0 SKS kebijakan UWG; tercatat di transkrip namun tidak dihitung dalam beban SKS kelulusan.</t>
+          <t>MKU-406 (Agama II) dan MKU-508 (Kewirausahaan II) = 0 SKS kebijakan UWG; tercatat di transkrip namun tidak dihitung dalam beban SKS kelulusan.</t>
         </is>
       </c>
     </row>
@@ -3167,14 +3167,14 @@
     <col width="10" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="13" t="inlineStr">
         <is>
           <t>SISTEKIN 2026 — Sheet 1: Cek List Kesiapan OBE</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1">
+    <row r="2" ht="16" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
           <t>SELF ASSESSMENT KESIAPAN IMPLEMENTASI MODUL OBE - S1 SISTEM DAN TEKNOLOGI INFORMASI 2026</t>
@@ -3208,7 +3208,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1">
+    <row r="4" ht="16" customHeight="1">
       <c r="A4" s="16" t="inlineStr">
         <is>
           <t>1</t>
@@ -3235,7 +3235,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1">
+    <row r="5" ht="16" customHeight="1">
       <c r="A5" s="17" t="inlineStr">
         <is>
           <t>2</t>
@@ -3262,7 +3262,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1">
+    <row r="6" ht="16" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
           <t>3</t>
@@ -3289,7 +3289,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1">
+    <row r="7" ht="16" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
           <t>4</t>
@@ -3316,7 +3316,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1">
+    <row r="8" ht="16" customHeight="1">
       <c r="A8" s="16" t="inlineStr">
         <is>
           <t>5</t>
@@ -3343,7 +3343,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1">
+    <row r="9" ht="16" customHeight="1">
       <c r="A9" s="17" t="inlineStr">
         <is>
           <t>6</t>
@@ -3370,7 +3370,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1">
+    <row r="10" ht="16" customHeight="1">
       <c r="A10" s="16" t="inlineStr">
         <is>
           <t>7</t>
@@ -3397,7 +3397,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1">
+    <row r="11" ht="16" customHeight="1">
       <c r="A11" s="17" t="inlineStr">
         <is>
           <t>8</t>
@@ -3424,7 +3424,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1">
+    <row r="12" ht="16" customHeight="1">
       <c r="A12" s="16" t="inlineStr">
         <is>
           <t>9</t>
@@ -3451,7 +3451,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1">
+    <row r="13" ht="16" customHeight="1">
       <c r="A13" s="17" t="inlineStr">
         <is>
           <t>10</t>
@@ -3478,7 +3478,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1">
+    <row r="14" ht="16" customHeight="1">
       <c r="A14" s="16" t="inlineStr">
         <is>
           <t>11</t>
@@ -3505,7 +3505,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="15" customHeight="1">
+    <row r="15" ht="16" customHeight="1">
       <c r="A15" s="17" t="inlineStr">
         <is>
           <t>12</t>
@@ -3532,7 +3532,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1">
+    <row r="16" ht="16" customHeight="1">
       <c r="A16" s="16" t="inlineStr">
         <is>
           <t>13</t>
@@ -3559,7 +3559,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="15" customHeight="1">
+    <row r="17" ht="16" customHeight="1">
       <c r="A17" s="17" t="inlineStr">
         <is>
           <t>14</t>
@@ -3586,7 +3586,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1">
+    <row r="18" ht="16" customHeight="1">
       <c r="A18" s="16" t="inlineStr">
         <is>
           <t>15</t>
@@ -3613,7 +3613,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1">
+    <row r="19" ht="16" customHeight="1">
       <c r="A19" s="17" t="inlineStr">
         <is>
           <t>16</t>
@@ -3640,7 +3640,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="15" customHeight="1">
+    <row r="20" ht="16" customHeight="1">
       <c r="A20" s="16" t="inlineStr">
         <is>
           <t>17</t>
@@ -3694,14 +3694,14 @@
     <col width="10" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="13" t="inlineStr">
         <is>
           <t>SISTEKIN 2026 — Sheet 2: Profil Lulusan (4 PL)</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1">
+    <row r="2" ht="16" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
           <t>PROFIL LULUSAN - S1 SISTEM DAN TEKNOLOGI INFORMASI 2026 (Dok. 002)</t>
@@ -3735,7 +3735,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1">
+    <row r="4" ht="16" customHeight="1">
       <c r="A4" s="16" t="inlineStr">
         <is>
           <t>1</t>
@@ -3762,7 +3762,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1">
+    <row r="5" ht="16" customHeight="1">
       <c r="A5" s="17" t="inlineStr">
         <is>
           <t>2</t>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1">
+    <row r="6" ht="16" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
           <t>3</t>
@@ -3816,7 +3816,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1">
+    <row r="7" ht="16" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
           <t>4</t>
@@ -3871,14 +3871,14 @@
     <col width="46" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="13" t="inlineStr">
         <is>
           <t>SISTEKIN 2026 — Sheet 3: CPL Prodi (14 CPL)</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1">
+    <row r="2" ht="16" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
           <t>CAPAIAN PEMBELAJARAN LULUSAN (CPL) - 14 OUTCOMES (S1 + KU1-3 + P1-4 + KK1-6)</t>
@@ -3922,7 +3922,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1">
+    <row r="4" ht="16" customHeight="1">
       <c r="A4" s="16" t="inlineStr">
         <is>
           <t>1</t>
@@ -3959,7 +3959,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1">
+    <row r="5" ht="16" customHeight="1">
       <c r="A5" s="17" t="inlineStr">
         <is>
           <t>2</t>
@@ -3996,7 +3996,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1">
+    <row r="6" ht="16" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
           <t>3</t>
@@ -4033,7 +4033,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1">
+    <row r="7" ht="16" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
           <t>4</t>
@@ -4070,7 +4070,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1">
+    <row r="8" ht="16" customHeight="1">
       <c r="A8" s="16" t="inlineStr">
         <is>
           <t>5</t>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1">
+    <row r="9" ht="16" customHeight="1">
       <c r="A9" s="17" t="inlineStr">
         <is>
           <t>6</t>
@@ -4144,7 +4144,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1">
+    <row r="10" ht="16" customHeight="1">
       <c r="A10" s="16" t="inlineStr">
         <is>
           <t>7</t>
@@ -4181,7 +4181,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1">
+    <row r="11" ht="16" customHeight="1">
       <c r="A11" s="17" t="inlineStr">
         <is>
           <t>8</t>
@@ -4218,7 +4218,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1">
+    <row r="12" ht="16" customHeight="1">
       <c r="A12" s="16" t="inlineStr">
         <is>
           <t>9</t>
@@ -4255,7 +4255,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1">
+    <row r="13" ht="16" customHeight="1">
       <c r="A13" s="17" t="inlineStr">
         <is>
           <t>10</t>
@@ -4292,7 +4292,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1">
+    <row r="14" ht="16" customHeight="1">
       <c r="A14" s="16" t="inlineStr">
         <is>
           <t>11</t>
@@ -4329,7 +4329,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="15" customHeight="1">
+    <row r="15" ht="16" customHeight="1">
       <c r="A15" s="17" t="inlineStr">
         <is>
           <t>12</t>
@@ -4366,7 +4366,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1">
+    <row r="16" ht="16" customHeight="1">
       <c r="A16" s="16" t="inlineStr">
         <is>
           <t>13</t>
@@ -4403,7 +4403,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="15" customHeight="1">
+    <row r="17" ht="16" customHeight="1">
       <c r="A17" s="17" t="inlineStr">
         <is>
           <t>14</t>
@@ -4469,14 +4469,14 @@
     <col width="40.25" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="13" t="inlineStr">
         <is>
           <t>SISTEKIN 2026 — Sheet 4: Matriks CPL - Profil Lulusan</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1">
+    <row r="2" ht="16" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
           <t>MATRIKS KETERKAITAN 14 CPL - 4 PROFIL LULUSAN (Dok. 004)</t>
@@ -4525,7 +4525,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1">
+    <row r="4" ht="16" customHeight="1">
       <c r="A4" s="16" t="inlineStr">
         <is>
           <t>1</t>
@@ -4567,7 +4567,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1">
+    <row r="5" ht="16" customHeight="1">
       <c r="A5" s="17" t="inlineStr">
         <is>
           <t>2</t>
@@ -4609,7 +4609,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1">
+    <row r="6" ht="16" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
           <t>3</t>
@@ -4651,7 +4651,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1">
+    <row r="7" ht="16" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
           <t>4</t>
@@ -4693,7 +4693,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1">
+    <row r="8" ht="16" customHeight="1">
       <c r="A8" s="16" t="inlineStr">
         <is>
           <t>5</t>
@@ -4735,7 +4735,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1">
+    <row r="9" ht="16" customHeight="1">
       <c r="A9" s="17" t="inlineStr">
         <is>
           <t>6</t>
@@ -4769,7 +4769,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1">
+    <row r="10" ht="16" customHeight="1">
       <c r="A10" s="16" t="inlineStr">
         <is>
           <t>7</t>
@@ -4799,7 +4799,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1">
+    <row r="11" ht="16" customHeight="1">
       <c r="A11" s="17" t="inlineStr">
         <is>
           <t>8</t>
@@ -4837,7 +4837,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1">
+    <row r="12" ht="16" customHeight="1">
       <c r="A12" s="16" t="inlineStr">
         <is>
           <t>9</t>
@@ -4867,7 +4867,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1">
+    <row r="13" ht="16" customHeight="1">
       <c r="A13" s="17" t="inlineStr">
         <is>
           <t>10</t>
@@ -4897,7 +4897,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1">
+    <row r="14" ht="16" customHeight="1">
       <c r="A14" s="16" t="inlineStr">
         <is>
           <t>11</t>
@@ -4927,7 +4927,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="15" customHeight="1">
+    <row r="15" ht="16" customHeight="1">
       <c r="A15" s="17" t="inlineStr">
         <is>
           <t>12</t>
@@ -4957,7 +4957,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1">
+    <row r="16" ht="16" customHeight="1">
       <c r="A16" s="16" t="inlineStr">
         <is>
           <t>13</t>
@@ -4987,7 +4987,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="15" customHeight="1">
+    <row r="17" ht="16" customHeight="1">
       <c r="A17" s="17" t="inlineStr">
         <is>
           <t>14</t>
@@ -5017,7 +5017,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1">
+    <row r="18" ht="16" customHeight="1">
       <c r="A18" s="20" t="inlineStr">
         <is>
           <t>Jumlah CPL per PL</t>
@@ -5092,14 +5092,14 @@
     <col width="40.25" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="13" t="inlineStr">
         <is>
           <t>SISTEKIN 2026 — Sheet 5: Matriks CPL - Mata Kuliah (67 MK Portofolio)</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1">
+    <row r="2" ht="16" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
           <t>MATRIKS PEMETAAN CPL - MATA KULIAH (55 MK PAKET / 146 SKS - PORTOFOLIO 67 MK / 182 SKS)</t>
@@ -5208,7 +5208,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1">
+    <row r="4" ht="16" customHeight="1">
       <c r="A4" s="21" t="inlineStr">
         <is>
           <t>A. MKWU - MATA KULIAH WAJIB UMUM (8 MK / 13 SKS)</t>
@@ -5234,7 +5234,7 @@
       <c r="S4" s="21" t="inlineStr"/>
       <c r="T4" s="21" t="inlineStr"/>
     </row>
-    <row r="5" ht="15" customHeight="1">
+    <row r="5" ht="16" customHeight="1">
       <c r="A5" s="17" t="inlineStr">
         <is>
           <t>1</t>
@@ -5284,7 +5284,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1">
+    <row r="6" ht="16" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
           <t>2</t>
@@ -5334,7 +5334,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1">
+    <row r="7" ht="16" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
           <t>3</t>
@@ -5384,7 +5384,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1">
+    <row r="8" ht="16" customHeight="1">
       <c r="A8" s="16" t="inlineStr">
         <is>
           <t>4</t>
@@ -5392,7 +5392,7 @@
       </c>
       <c r="B8" s="16" t="inlineStr">
         <is>
-          <t>MKU-202</t>
+          <t>MKU-204</t>
         </is>
       </c>
       <c r="C8" s="16" t="inlineStr">
@@ -5434,7 +5434,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1">
+    <row r="9" ht="16" customHeight="1">
       <c r="A9" s="17" t="inlineStr">
         <is>
           <t>5</t>
@@ -5442,12 +5442,12 @@
       </c>
       <c r="B9" s="17" t="inlineStr">
         <is>
-          <t>MKU-201</t>
+          <t>MKU-405</t>
         </is>
       </c>
       <c r="C9" s="17" t="inlineStr">
         <is>
-          <t>Pendidikan Kewarganegaraan</t>
+          <t>Kewarganegaraan</t>
         </is>
       </c>
       <c r="D9" s="17" t="inlineStr">
@@ -5484,7 +5484,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1">
+    <row r="10" ht="16" customHeight="1">
       <c r="A10" s="16" t="inlineStr">
         <is>
           <t>6</t>
@@ -5492,7 +5492,7 @@
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>MKU-401A</t>
+          <t>MKU-406</t>
         </is>
       </c>
       <c r="C10" s="16" t="inlineStr">
@@ -5534,7 +5534,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1">
+    <row r="11" ht="16" customHeight="1">
       <c r="A11" s="17" t="inlineStr">
         <is>
           <t>7</t>
@@ -5542,7 +5542,7 @@
       </c>
       <c r="B11" s="17" t="inlineStr">
         <is>
-          <t>MKU-402</t>
+          <t>MKU-508</t>
         </is>
       </c>
       <c r="C11" s="17" t="inlineStr">
@@ -5584,7 +5584,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1">
+    <row r="12" ht="16" customHeight="1">
       <c r="A12" s="16" t="inlineStr">
         <is>
           <t>8</t>
@@ -5592,12 +5592,12 @@
       </c>
       <c r="B12" s="16" t="inlineStr">
         <is>
-          <t>MKU-203</t>
+          <t>MKU-507</t>
         </is>
       </c>
       <c r="C12" s="16" t="inlineStr">
         <is>
-          <t>KPM (Kuliah Pengabdian Masyarakat)</t>
+          <t>KPM (Kuliah Pengabdian Kepada Masyarakat)</t>
         </is>
       </c>
       <c r="D12" s="16" t="inlineStr">
@@ -5638,7 +5638,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1">
+    <row r="13" ht="16" customHeight="1">
       <c r="A13" s="21" t="inlineStr">
         <is>
           <t>B. MK FSTI - MATA KULIAH WAJIB FAKULTAS (14 MK / 38 SKS)</t>
@@ -5664,7 +5664,7 @@
       <c r="S13" s="21" t="inlineStr"/>
       <c r="T13" s="21" t="inlineStr"/>
     </row>
-    <row r="14" ht="15" customHeight="1">
+    <row r="14" ht="16" customHeight="1">
       <c r="A14" s="16" t="inlineStr">
         <is>
           <t>9</t>
@@ -5714,7 +5714,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="15" customHeight="1">
+    <row r="15" ht="16" customHeight="1">
       <c r="A15" s="17" t="inlineStr">
         <is>
           <t>10</t>
@@ -5768,7 +5768,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1">
+    <row r="16" ht="16" customHeight="1">
       <c r="A16" s="16" t="inlineStr">
         <is>
           <t>11</t>
@@ -5822,7 +5822,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="15" customHeight="1">
+    <row r="17" ht="16" customHeight="1">
       <c r="A17" s="17" t="inlineStr">
         <is>
           <t>12</t>
@@ -5872,7 +5872,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1">
+    <row r="18" ht="16" customHeight="1">
       <c r="A18" s="16" t="inlineStr">
         <is>
           <t>13</t>
@@ -5922,7 +5922,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1">
+    <row r="19" ht="16" customHeight="1">
       <c r="A19" s="17" t="inlineStr">
         <is>
           <t>14</t>
@@ -5976,7 +5976,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="15" customHeight="1">
+    <row r="20" ht="16" customHeight="1">
       <c r="A20" s="16" t="inlineStr">
         <is>
           <t>15</t>
@@ -6030,7 +6030,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1">
+    <row r="21" ht="16" customHeight="1">
       <c r="A21" s="17" t="inlineStr">
         <is>
           <t>16</t>
@@ -6084,7 +6084,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="15" customHeight="1">
+    <row r="22" ht="16" customHeight="1">
       <c r="A22" s="16" t="inlineStr">
         <is>
           <t>17</t>
@@ -6134,7 +6134,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1">
+    <row r="23" ht="16" customHeight="1">
       <c r="A23" s="17" t="inlineStr">
         <is>
           <t>18</t>
@@ -6220,7 +6220,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="15" customHeight="1">
+    <row r="24" ht="16" customHeight="1">
       <c r="A24" s="16" t="inlineStr">
         <is>
           <t>19</t>
@@ -6278,7 +6278,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="15" customHeight="1">
+    <row r="25" ht="16" customHeight="1">
       <c r="A25" s="17" t="inlineStr">
         <is>
           <t>20</t>
@@ -6348,7 +6348,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="15" customHeight="1">
+    <row r="26" ht="16" customHeight="1">
       <c r="A26" s="16" t="inlineStr">
         <is>
           <t>21</t>
@@ -6406,7 +6406,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="15" customHeight="1">
+    <row r="27" ht="16" customHeight="1">
       <c r="A27" s="17" t="inlineStr">
         <is>
           <t>22</t>
@@ -6508,7 +6508,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="15" customHeight="1">
+    <row r="28" ht="16" customHeight="1">
       <c r="A28" s="21" t="inlineStr">
         <is>
           <t>C. MK CORE STI - MATA KULIAH INTI PROGRAM STUDI (27 MK / 77 SKS)</t>
@@ -6534,7 +6534,7 @@
       <c r="S28" s="21" t="inlineStr"/>
       <c r="T28" s="21" t="inlineStr"/>
     </row>
-    <row r="29" ht="15" customHeight="1">
+    <row r="29" ht="16" customHeight="1">
       <c r="A29" s="17" t="inlineStr">
         <is>
           <t>23</t>
@@ -6584,7 +6584,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="15" customHeight="1">
+    <row r="30" ht="16" customHeight="1">
       <c r="A30" s="16" t="inlineStr">
         <is>
           <t>24</t>
@@ -6634,7 +6634,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="15" customHeight="1">
+    <row r="31" ht="16" customHeight="1">
       <c r="A31" s="17" t="inlineStr">
         <is>
           <t>25</t>
@@ -6688,7 +6688,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="15" customHeight="1">
+    <row r="32" ht="16" customHeight="1">
       <c r="A32" s="16" t="inlineStr">
         <is>
           <t>26</t>
@@ -6742,7 +6742,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="15" customHeight="1">
+    <row r="33" ht="16" customHeight="1">
       <c r="A33" s="17" t="inlineStr">
         <is>
           <t>27</t>
@@ -6792,7 +6792,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="15" customHeight="1">
+    <row r="34" ht="16" customHeight="1">
       <c r="A34" s="16" t="inlineStr">
         <is>
           <t>28</t>
@@ -6850,7 +6850,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="15" customHeight="1">
+    <row r="35" ht="16" customHeight="1">
       <c r="A35" s="17" t="inlineStr">
         <is>
           <t>29</t>
@@ -6904,7 +6904,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="15" customHeight="1">
+    <row r="36" ht="16" customHeight="1">
       <c r="A36" s="16" t="inlineStr">
         <is>
           <t>30</t>
@@ -6954,7 +6954,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="15" customHeight="1">
+    <row r="37" ht="16" customHeight="1">
       <c r="A37" s="17" t="inlineStr">
         <is>
           <t>31</t>
@@ -7012,7 +7012,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="15" customHeight="1">
+    <row r="38" ht="16" customHeight="1">
       <c r="A38" s="16" t="inlineStr">
         <is>
           <t>32</t>
@@ -7066,7 +7066,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="15" customHeight="1">
+    <row r="39" ht="16" customHeight="1">
       <c r="A39" s="17" t="inlineStr">
         <is>
           <t>33</t>
@@ -7120,7 +7120,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="15" customHeight="1">
+    <row r="40" ht="16" customHeight="1">
       <c r="A40" s="16" t="inlineStr">
         <is>
           <t>34</t>
@@ -7174,7 +7174,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="15" customHeight="1">
+    <row r="41" ht="16" customHeight="1">
       <c r="A41" s="17" t="inlineStr">
         <is>
           <t>35</t>
@@ -7232,7 +7232,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="15" customHeight="1">
+    <row r="42" ht="16" customHeight="1">
       <c r="A42" s="16" t="inlineStr">
         <is>
           <t>36</t>
@@ -7286,7 +7286,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="15" customHeight="1">
+    <row r="43" ht="16" customHeight="1">
       <c r="A43" s="17" t="inlineStr">
         <is>
           <t>37</t>
@@ -7340,7 +7340,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="15" customHeight="1">
+    <row r="44" ht="16" customHeight="1">
       <c r="A44" s="16" t="inlineStr">
         <is>
           <t>38</t>
@@ -7394,7 +7394,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="15" customHeight="1">
+    <row r="45" ht="16" customHeight="1">
       <c r="A45" s="17" t="inlineStr">
         <is>
           <t>39</t>
@@ -7448,7 +7448,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="15" customHeight="1">
+    <row r="46" ht="16" customHeight="1">
       <c r="A46" s="16" t="inlineStr">
         <is>
           <t>40</t>
@@ -7502,7 +7502,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="15" customHeight="1">
+    <row r="47" ht="16" customHeight="1">
       <c r="A47" s="17" t="inlineStr">
         <is>
           <t>41</t>
@@ -7556,7 +7556,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="15" customHeight="1">
+    <row r="48" ht="16" customHeight="1">
       <c r="A48" s="16" t="inlineStr">
         <is>
           <t>42</t>
@@ -7610,7 +7610,7 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="15" customHeight="1">
+    <row r="49" ht="16" customHeight="1">
       <c r="A49" s="17" t="inlineStr">
         <is>
           <t>43</t>
@@ -7664,7 +7664,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="15" customHeight="1">
+    <row r="50" ht="16" customHeight="1">
       <c r="A50" s="16" t="inlineStr">
         <is>
           <t>44</t>
@@ -7714,7 +7714,7 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="15" customHeight="1">
+    <row r="51" ht="16" customHeight="1">
       <c r="A51" s="17" t="inlineStr">
         <is>
           <t>45</t>
@@ -7768,7 +7768,7 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="15" customHeight="1">
+    <row r="52" ht="16" customHeight="1">
       <c r="A52" s="16" t="inlineStr">
         <is>
           <t>46</t>
@@ -7822,7 +7822,7 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="15" customHeight="1">
+    <row r="53" ht="16" customHeight="1">
       <c r="A53" s="17" t="inlineStr">
         <is>
           <t>47</t>
@@ -7880,7 +7880,7 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="15" customHeight="1">
+    <row r="54" ht="16" customHeight="1">
       <c r="A54" s="16" t="inlineStr">
         <is>
           <t>48</t>
@@ -7934,7 +7934,7 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="15" customHeight="1">
+    <row r="55" ht="16" customHeight="1">
       <c r="A55" s="17" t="inlineStr">
         <is>
           <t>49</t>
@@ -7984,7 +7984,7 @@
         </is>
       </c>
     </row>
-    <row r="56" ht="15" customHeight="1">
+    <row r="56" ht="16" customHeight="1">
       <c r="A56" s="21" t="inlineStr">
         <is>
           <t>D. MK PILIHAN P1: INTEGRATED SMART SYSTEMS (6 MK / 18 SKS)</t>
@@ -8010,7 +8010,7 @@
       <c r="S56" s="21" t="inlineStr"/>
       <c r="T56" s="21" t="inlineStr"/>
     </row>
-    <row r="57" ht="15" customHeight="1">
+    <row r="57" ht="16" customHeight="1">
       <c r="A57" s="17" t="inlineStr">
         <is>
           <t>50</t>
@@ -8064,7 +8064,7 @@
         </is>
       </c>
     </row>
-    <row r="58" ht="15" customHeight="1">
+    <row r="58" ht="16" customHeight="1">
       <c r="A58" s="16" t="inlineStr">
         <is>
           <t>51</t>
@@ -8118,7 +8118,7 @@
         </is>
       </c>
     </row>
-    <row r="59" ht="15" customHeight="1">
+    <row r="59" ht="16" customHeight="1">
       <c r="A59" s="17" t="inlineStr">
         <is>
           <t>52</t>
@@ -8168,7 +8168,7 @@
         </is>
       </c>
     </row>
-    <row r="60" ht="15" customHeight="1">
+    <row r="60" ht="16" customHeight="1">
       <c r="A60" s="16" t="inlineStr">
         <is>
           <t>53</t>
@@ -8222,7 +8222,7 @@
         </is>
       </c>
     </row>
-    <row r="61" ht="15" customHeight="1">
+    <row r="61" ht="16" customHeight="1">
       <c r="A61" s="17" t="inlineStr">
         <is>
           <t>54</t>
@@ -8272,7 +8272,7 @@
         </is>
       </c>
     </row>
-    <row r="62" ht="15" customHeight="1">
+    <row r="62" ht="16" customHeight="1">
       <c r="A62" s="16" t="inlineStr">
         <is>
           <t>55</t>
@@ -8326,7 +8326,7 @@
         </is>
       </c>
     </row>
-    <row r="63" ht="15" customHeight="1">
+    <row r="63" ht="16" customHeight="1">
       <c r="A63" s="21" t="inlineStr">
         <is>
           <t>E. MK PILIHAN P2: CLOUD INFRASTRUCTURE &amp; CYBERSECURITY (6 MK / 18 SKS)</t>
@@ -8352,7 +8352,7 @@
       <c r="S63" s="21" t="inlineStr"/>
       <c r="T63" s="21" t="inlineStr"/>
     </row>
-    <row r="64" ht="15" customHeight="1">
+    <row r="64" ht="16" customHeight="1">
       <c r="A64" s="16" t="inlineStr">
         <is>
           <t>56</t>
@@ -8410,7 +8410,7 @@
         </is>
       </c>
     </row>
-    <row r="65" ht="15" customHeight="1">
+    <row r="65" ht="16" customHeight="1">
       <c r="A65" s="17" t="inlineStr">
         <is>
           <t>57</t>
@@ -8464,7 +8464,7 @@
         </is>
       </c>
     </row>
-    <row r="66" ht="15" customHeight="1">
+    <row r="66" ht="16" customHeight="1">
       <c r="A66" s="16" t="inlineStr">
         <is>
           <t>58</t>
@@ -8518,7 +8518,7 @@
         </is>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1">
+    <row r="67" ht="16" customHeight="1">
       <c r="A67" s="17" t="inlineStr">
         <is>
           <t>59</t>
@@ -8568,7 +8568,7 @@
         </is>
       </c>
     </row>
-    <row r="68" ht="15" customHeight="1">
+    <row r="68" ht="16" customHeight="1">
       <c r="A68" s="16" t="inlineStr">
         <is>
           <t>60</t>
@@ -8622,7 +8622,7 @@
         </is>
       </c>
     </row>
-    <row r="69" ht="15" customHeight="1">
+    <row r="69" ht="16" customHeight="1">
       <c r="A69" s="17" t="inlineStr">
         <is>
           <t>61</t>
@@ -8676,7 +8676,7 @@
         </is>
       </c>
     </row>
-    <row r="70" ht="15" customHeight="1">
+    <row r="70" ht="16" customHeight="1">
       <c r="A70" s="21" t="inlineStr">
         <is>
           <t>F. MK PILIHAN P3: DIGITAL PLATFORM ENGINEERING (6 MK / 18 SKS)</t>
@@ -8702,7 +8702,7 @@
       <c r="S70" s="21" t="inlineStr"/>
       <c r="T70" s="21" t="inlineStr"/>
     </row>
-    <row r="71" ht="15" customHeight="1">
+    <row r="71" ht="16" customHeight="1">
       <c r="A71" s="17" t="inlineStr">
         <is>
           <t>62</t>
@@ -8752,7 +8752,7 @@
         </is>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1">
+    <row r="72" ht="16" customHeight="1">
       <c r="A72" s="16" t="inlineStr">
         <is>
           <t>63</t>
@@ -8802,7 +8802,7 @@
         </is>
       </c>
     </row>
-    <row r="73" ht="15" customHeight="1">
+    <row r="73" ht="16" customHeight="1">
       <c r="A73" s="17" t="inlineStr">
         <is>
           <t>64</t>
@@ -8852,7 +8852,7 @@
         </is>
       </c>
     </row>
-    <row r="74" ht="15" customHeight="1">
+    <row r="74" ht="16" customHeight="1">
       <c r="A74" s="16" t="inlineStr">
         <is>
           <t>65</t>
@@ -8902,7 +8902,7 @@
         </is>
       </c>
     </row>
-    <row r="75" ht="15" customHeight="1">
+    <row r="75" ht="16" customHeight="1">
       <c r="A75" s="17" t="inlineStr">
         <is>
           <t>66</t>
@@ -8952,7 +8952,7 @@
         </is>
       </c>
     </row>
-    <row r="76" ht="15" customHeight="1">
+    <row r="76" ht="16" customHeight="1">
       <c r="A76" s="16" t="inlineStr">
         <is>
           <t>67</t>
@@ -9002,7 +9002,7 @@
         </is>
       </c>
     </row>
-    <row r="77" ht="15" customHeight="1">
+    <row r="77" ht="16" customHeight="1">
       <c r="A77" s="20" t="inlineStr">
         <is>
           <t>Jumlah MK Pendukung tiap CPL</t>
@@ -9116,14 +9116,14 @@
     <col width="69" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="13" t="inlineStr">
         <is>
           <t>SISTEKIN 2026 — Sheet 6: Organisasi Mata Kuliah Per Semester</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1">
+    <row r="2" ht="16" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
           <t>ORGANISASI MATA KULIAH - KURIKULUM SISTEKIN 2026 (Dok. 005)</t>
@@ -9167,7 +9167,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1">
+    <row r="4" ht="16" customHeight="1">
       <c r="A4" s="16" t="inlineStr">
         <is>
           <t>1</t>
@@ -9204,7 +9204,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1">
+    <row r="5" ht="16" customHeight="1">
       <c r="A5" s="17" t="inlineStr">
         <is>
           <t>2</t>
@@ -9227,7 +9227,7 @@
       </c>
       <c r="E5" s="17" t="inlineStr">
         <is>
-          <t>STI-201 Matematika Diskrit (3) / STI-202 Aljabar Linear (3) / FST-203 Struktur Data &amp; Algoritma (3) / FST-204 Pengantar AI &amp; Data (2) / FST-205 Basic English (2) / FST-206 Etika &amp; Hukum Digital (2) / FST-207 Basis Data (3) / MKU-202 Kewirausahaan I (2)</t>
+          <t>STI-201 Matematika Diskrit (3) / STI-202 Aljabar Linear (3) / FST-203 Struktur Data &amp; Algoritma (3) / FST-204 Pengantar AI &amp; Data (2) / FST-205 Basic English (2) / FST-206 Etika &amp; Hukum Digital (2) / FST-207 Basis Data (3) / MKU-204 Kewirausahaan I (2)</t>
         </is>
       </c>
       <c r="F5" s="19" t="inlineStr">
@@ -9241,7 +9241,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1">
+    <row r="6" ht="16" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
           <t>3</t>
@@ -9278,7 +9278,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1">
+    <row r="7" ht="16" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
           <t>4</t>
@@ -9301,7 +9301,7 @@
       </c>
       <c r="E7" s="17" t="inlineStr">
         <is>
-          <t>STI-401 Machine Learning (3) / STI-402 DW &amp; BI (3) / STI-404 Cloud (3) / STI-405 Dasar Keamanan (2) / STI-407 Web Back End (3) / FST-408 Statistika (3) / FST-409 Manajemen Sains (2) / MKU-201 KWN (2) / MKU-401A Agama II (0)</t>
+          <t>STI-401 Machine Learning (3) / STI-402 DW &amp; BI (3) / STI-404 Cloud (3) / STI-405 Dasar Keamanan (2) / STI-407 Web Back End (3) / FST-408 Statistika (3) / FST-409 Manajemen Sains (2) / MKU-405 KWN (2) / MKU-406 Agama II (0)</t>
         </is>
       </c>
       <c r="F7" s="19" t="inlineStr">
@@ -9311,11 +9311,11 @@
       </c>
       <c r="G7" s="19" t="inlineStr">
         <is>
-          <t>STI-405 = 2 SKS Teori. MKU-401A = 0 SKS kebijakan UWG</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="15" customHeight="1">
+          <t>STI-405 = 2 SKS Teori. MKU-406 = 0 SKS kebijakan UWG</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="16" customHeight="1">
       <c r="A8" s="16" t="inlineStr">
         <is>
           <t>5</t>
@@ -9338,7 +9338,7 @@
       </c>
       <c r="E8" s="16" t="inlineStr">
         <is>
-          <t>STI-501 Deep Learning (3) / STI-503 Data Mining (3) / STI-504 IoT (3) / STI-505 Mobile App (3) / STI-506 Manpro TI (3) / MKU-203 KPM (3) / MK Pilihan 1 (3) / MKU-402 KWU II (0)</t>
+          <t>STI-501 Deep Learning (3) / STI-503 Data Mining (3) / STI-504 IoT (3) / STI-505 Mobile App (3) / STI-506 Manpro TI (3) / MKU-507 KPM (3) / MK Pilihan 1 (3) / MKU-508 KWU II (0)</t>
         </is>
       </c>
       <c r="F8" s="18" t="inlineStr">
@@ -9348,11 +9348,11 @@
       </c>
       <c r="G8" s="18" t="inlineStr">
         <is>
-          <t>6 MK Wajib (18 SKS) + 1 MK Pilihan (3 SKS). MKU-402 = 0 SKS kebijakan UWG</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="15" customHeight="1">
+          <t>6 MK Wajib (18 SKS) + 1 MK Pilihan (3 SKS). MKU-508 = 0 SKS kebijakan UWG</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="16" customHeight="1">
       <c r="A9" s="17" t="inlineStr">
         <is>
           <t>6</t>
@@ -9389,7 +9389,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1">
+    <row r="10" ht="16" customHeight="1">
       <c r="A10" s="16" t="inlineStr">
         <is>
           <t>7</t>
@@ -9426,7 +9426,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1">
+    <row r="11" ht="16" customHeight="1">
       <c r="A11" s="17" t="inlineStr">
         <is>
           <t>8</t>
@@ -9463,7 +9463,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1">
+    <row r="12" ht="16" customHeight="1">
       <c r="A12" s="20" t="inlineStr">
         <is>
           <t>TOTAL</t>
@@ -9536,14 +9536,14 @@
     <col width="10" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="13" t="inlineStr">
         <is>
           <t>SISTEKIN 2026 — Sheet 7: Peta Pemenuhan CPL (Level I-R-M)</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1">
+    <row r="2" ht="16" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
           <t>PETA PEMENUHAN CPL OLEH MATA KULIAH - LEVEL I/R/M (Dok. 004)</t>
@@ -9647,7 +9647,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1">
+    <row r="4" ht="16" customHeight="1">
       <c r="A4" s="16" t="inlineStr">
         <is>
           <t>MKU-101</t>
@@ -9692,7 +9692,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1">
+    <row r="5" ht="16" customHeight="1">
       <c r="A5" s="17" t="inlineStr">
         <is>
           <t>MKU-102</t>
@@ -9737,7 +9737,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1">
+    <row r="6" ht="16" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
           <t>MKU-103</t>
@@ -9782,7 +9782,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1">
+    <row r="7" ht="16" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
           <t>FST-101</t>
@@ -9827,7 +9827,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1">
+    <row r="8" ht="16" customHeight="1">
       <c r="A8" s="16" t="inlineStr">
         <is>
           <t>FST-102</t>
@@ -9876,7 +9876,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1">
+    <row r="9" ht="16" customHeight="1">
       <c r="A9" s="17" t="inlineStr">
         <is>
           <t>STI-101</t>
@@ -9921,7 +9921,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1">
+    <row r="10" ht="16" customHeight="1">
       <c r="A10" s="16" t="inlineStr">
         <is>
           <t>STI-102</t>
@@ -9966,7 +9966,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1">
+    <row r="11" ht="16" customHeight="1">
       <c r="A11" s="17" t="inlineStr">
         <is>
           <t>STI-103</t>
@@ -10015,10 +10015,10 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1">
+    <row r="12" ht="16" customHeight="1">
       <c r="A12" s="16" t="inlineStr">
         <is>
-          <t>MKU-202</t>
+          <t>MKU-204</t>
         </is>
       </c>
       <c r="B12" s="16" t="inlineStr">
@@ -10060,7 +10060,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1">
+    <row r="13" ht="16" customHeight="1">
       <c r="A13" s="17" t="inlineStr">
         <is>
           <t>STI-201</t>
@@ -10109,7 +10109,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1">
+    <row r="14" ht="16" customHeight="1">
       <c r="A14" s="16" t="inlineStr">
         <is>
           <t>STI-202</t>
@@ -10154,7 +10154,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="15" customHeight="1">
+    <row r="15" ht="16" customHeight="1">
       <c r="A15" s="17" t="inlineStr">
         <is>
           <t>FST-203</t>
@@ -10203,7 +10203,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1">
+    <row r="16" ht="16" customHeight="1">
       <c r="A16" s="16" t="inlineStr">
         <is>
           <t>FST-204</t>
@@ -10248,7 +10248,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="15" customHeight="1">
+    <row r="17" ht="16" customHeight="1">
       <c r="A17" s="17" t="inlineStr">
         <is>
           <t>FST-205</t>
@@ -10293,7 +10293,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1">
+    <row r="18" ht="16" customHeight="1">
       <c r="A18" s="16" t="inlineStr">
         <is>
           <t>FST-206</t>
@@ -10342,7 +10342,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1">
+    <row r="19" ht="16" customHeight="1">
       <c r="A19" s="17" t="inlineStr">
         <is>
           <t>FST-207</t>
@@ -10391,7 +10391,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="15" customHeight="1">
+    <row r="20" ht="16" customHeight="1">
       <c r="A20" s="16" t="inlineStr">
         <is>
           <t>STI-301</t>
@@ -10444,7 +10444,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1">
+    <row r="21" ht="16" customHeight="1">
       <c r="A21" s="17" t="inlineStr">
         <is>
           <t>STI-302</t>
@@ -10493,7 +10493,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="15" customHeight="1">
+    <row r="22" ht="16" customHeight="1">
       <c r="A22" s="16" t="inlineStr">
         <is>
           <t>STI-303</t>
@@ -10538,7 +10538,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1">
+    <row r="23" ht="16" customHeight="1">
       <c r="A23" s="17" t="inlineStr">
         <is>
           <t>STI-304</t>
@@ -10591,7 +10591,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="15" customHeight="1">
+    <row r="24" ht="16" customHeight="1">
       <c r="A24" s="16" t="inlineStr">
         <is>
           <t>STI-305</t>
@@ -10640,7 +10640,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="15" customHeight="1">
+    <row r="25" ht="16" customHeight="1">
       <c r="A25" s="17" t="inlineStr">
         <is>
           <t>STI-306</t>
@@ -10689,7 +10689,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="15" customHeight="1">
+    <row r="26" ht="16" customHeight="1">
       <c r="A26" s="16" t="inlineStr">
         <is>
           <t>STI-307</t>
@@ -10738,7 +10738,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="15" customHeight="1">
+    <row r="27" ht="16" customHeight="1">
       <c r="A27" s="17" t="inlineStr">
         <is>
           <t>STI-401</t>
@@ -10791,7 +10791,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="15" customHeight="1">
+    <row r="28" ht="16" customHeight="1">
       <c r="A28" s="16" t="inlineStr">
         <is>
           <t>STI-402</t>
@@ -10840,7 +10840,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="15" customHeight="1">
+    <row r="29" ht="16" customHeight="1">
       <c r="A29" s="17" t="inlineStr">
         <is>
           <t>STI-404</t>
@@ -10889,7 +10889,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="15" customHeight="1">
+    <row r="30" ht="16" customHeight="1">
       <c r="A30" s="16" t="inlineStr">
         <is>
           <t>STI-405</t>
@@ -10938,7 +10938,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="15" customHeight="1">
+    <row r="31" ht="16" customHeight="1">
       <c r="A31" s="17" t="inlineStr">
         <is>
           <t>STI-407</t>
@@ -10987,7 +10987,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="15" customHeight="1">
+    <row r="32" ht="16" customHeight="1">
       <c r="A32" s="16" t="inlineStr">
         <is>
           <t>FST-408</t>
@@ -11036,7 +11036,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="15" customHeight="1">
+    <row r="33" ht="16" customHeight="1">
       <c r="A33" s="17" t="inlineStr">
         <is>
           <t>FST-409</t>
@@ -11081,7 +11081,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="15" customHeight="1">
+    <row r="34" ht="16" customHeight="1">
       <c r="A34" s="16" t="inlineStr">
         <is>
           <t>STI-501</t>
@@ -11130,7 +11130,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="15" customHeight="1">
+    <row r="35" ht="16" customHeight="1">
       <c r="A35" s="17" t="inlineStr">
         <is>
           <t>STI-503</t>
@@ -11179,7 +11179,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="15" customHeight="1">
+    <row r="36" ht="16" customHeight="1">
       <c r="A36" s="16" t="inlineStr">
         <is>
           <t>STI-504</t>
@@ -11228,7 +11228,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="15" customHeight="1">
+    <row r="37" ht="16" customHeight="1">
       <c r="A37" s="17" t="inlineStr">
         <is>
           <t>STI-505</t>
@@ -11277,7 +11277,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="15" customHeight="1">
+    <row r="38" ht="16" customHeight="1">
       <c r="A38" s="16" t="inlineStr">
         <is>
           <t>STI-506</t>
@@ -11322,10 +11322,10 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="15" customHeight="1">
+    <row r="39" ht="16" customHeight="1">
       <c r="A39" s="17" t="inlineStr">
         <is>
-          <t>MKU-203</t>
+          <t>MKU-507</t>
         </is>
       </c>
       <c r="B39" s="17" t="inlineStr">
@@ -11371,7 +11371,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="15" customHeight="1">
+    <row r="40" ht="16" customHeight="1">
       <c r="A40" s="16" t="inlineStr">
         <is>
           <t>STI-601</t>
@@ -11420,7 +11420,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="15" customHeight="1">
+    <row r="41" ht="16" customHeight="1">
       <c r="A41" s="17" t="inlineStr">
         <is>
           <t>STI-602</t>
@@ -11469,7 +11469,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="15" customHeight="1">
+    <row r="42" ht="16" customHeight="1">
       <c r="A42" s="16" t="inlineStr">
         <is>
           <t>STI-603</t>
@@ -11522,7 +11522,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="15" customHeight="1">
+    <row r="43" ht="16" customHeight="1">
       <c r="A43" s="17" t="inlineStr">
         <is>
           <t>STI-604</t>
@@ -11571,7 +11571,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="15" customHeight="1">
+    <row r="44" ht="16" customHeight="1">
       <c r="A44" s="16" t="inlineStr">
         <is>
           <t>FST-611</t>
@@ -11624,7 +11624,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="15" customHeight="1">
+    <row r="45" ht="16" customHeight="1">
       <c r="A45" s="17" t="inlineStr">
         <is>
           <t>STI-701</t>
@@ -11669,7 +11669,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="15" customHeight="1">
+    <row r="46" ht="16" customHeight="1">
       <c r="A46" s="16" t="inlineStr">
         <is>
           <t>FST-610</t>
@@ -11750,7 +11750,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="15" customHeight="1">
+    <row r="47" ht="16" customHeight="1">
       <c r="A47" s="17" t="inlineStr">
         <is>
           <t>FST-612</t>
@@ -11815,7 +11815,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="15" customHeight="1">
+    <row r="48" ht="16" customHeight="1">
       <c r="A48" s="16" t="inlineStr">
         <is>
           <t>FST-613</t>
@@ -11868,7 +11868,7 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="15" customHeight="1">
+    <row r="49" ht="16" customHeight="1">
       <c r="A49" s="17" t="inlineStr">
         <is>
           <t>FST-714</t>
@@ -11965,7 +11965,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="15" customHeight="1">
+    <row r="50" ht="16" customHeight="1">
       <c r="A50" s="20" t="inlineStr">
         <is>
           <t>Jumlah I</t>
@@ -12046,7 +12046,7 @@
       </c>
       <c r="S50" s="20" t="inlineStr"/>
     </row>
-    <row r="51" ht="15" customHeight="1">
+    <row r="51" ht="16" customHeight="1">
       <c r="A51" s="20" t="inlineStr">
         <is>
           <t>Jumlah R</t>
@@ -12127,7 +12127,7 @@
       </c>
       <c r="S51" s="20" t="inlineStr"/>
     </row>
-    <row r="52" ht="15" customHeight="1">
+    <row r="52" ht="16" customHeight="1">
       <c r="A52" s="20" t="inlineStr">
         <is>
           <t>Jumlah M</t>
@@ -12239,14 +12239,14 @@
     <col width="10.35" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="13" t="inlineStr">
         <is>
           <t>SISTEKIN 2026 — Sheet 8: Penurunan CPL ke CPMK &amp; Sub-CPMK (6 MK Penciri)</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1">
+    <row r="2" ht="16" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
           <t>PENURUNAN CPL -&gt; CPMK -&gt; SUB-CPMK -&gt; EVALUASI - 6 MK PENCIRI SISTEKIN 2026 (Dok. 007)</t>
@@ -12305,7 +12305,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1">
+    <row r="4" ht="16" customHeight="1">
       <c r="A4" s="16" t="inlineStr">
         <is>
           <t>STI-601</t>
@@ -12357,7 +12357,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1">
+    <row r="5" ht="16" customHeight="1">
       <c r="A5" s="17" t="inlineStr">
         <is>
           <t>STI-601</t>
@@ -12409,7 +12409,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1">
+    <row r="6" ht="16" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
           <t>STI-601</t>
@@ -12461,7 +12461,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1">
+    <row r="7" ht="16" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
           <t>STI-601</t>
@@ -12513,7 +12513,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1">
+    <row r="8" ht="16" customHeight="1">
       <c r="A8" s="16" t="inlineStr">
         <is>
           <t>STI-401</t>
@@ -12565,7 +12565,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1">
+    <row r="9" ht="16" customHeight="1">
       <c r="A9" s="17" t="inlineStr">
         <is>
           <t>STI-401</t>
@@ -12617,7 +12617,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1">
+    <row r="10" ht="16" customHeight="1">
       <c r="A10" s="16" t="inlineStr">
         <is>
           <t>STI-401</t>
@@ -12669,7 +12669,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1">
+    <row r="11" ht="16" customHeight="1">
       <c r="A11" s="17" t="inlineStr">
         <is>
           <t>STI-401</t>
@@ -12721,7 +12721,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1">
+    <row r="12" ht="16" customHeight="1">
       <c r="A12" s="16" t="inlineStr">
         <is>
           <t>STI-504</t>
@@ -12773,7 +12773,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1">
+    <row r="13" ht="16" customHeight="1">
       <c r="A13" s="17" t="inlineStr">
         <is>
           <t>STI-504</t>
@@ -12825,7 +12825,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1">
+    <row r="14" ht="16" customHeight="1">
       <c r="A14" s="16" t="inlineStr">
         <is>
           <t>STI-504</t>
@@ -12877,7 +12877,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="15" customHeight="1">
+    <row r="15" ht="16" customHeight="1">
       <c r="A15" s="17" t="inlineStr">
         <is>
           <t>STI-303</t>
@@ -12929,7 +12929,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1">
+    <row r="16" ht="16" customHeight="1">
       <c r="A16" s="16" t="inlineStr">
         <is>
           <t>STI-303</t>
@@ -12981,7 +12981,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="15" customHeight="1">
+    <row r="17" ht="16" customHeight="1">
       <c r="A17" s="17" t="inlineStr">
         <is>
           <t>STI-303</t>
@@ -13033,7 +13033,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1">
+    <row r="18" ht="16" customHeight="1">
       <c r="A18" s="16" t="inlineStr">
         <is>
           <t>STI-604</t>
@@ -13085,7 +13085,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1">
+    <row r="19" ht="16" customHeight="1">
       <c r="A19" s="17" t="inlineStr">
         <is>
           <t>STI-604</t>
@@ -13137,7 +13137,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="15" customHeight="1">
+    <row r="20" ht="16" customHeight="1">
       <c r="A20" s="16" t="inlineStr">
         <is>
           <t>STI-604</t>
@@ -13189,7 +13189,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1">
+    <row r="21" ht="16" customHeight="1">
       <c r="A21" s="17" t="inlineStr">
         <is>
           <t>STI-603</t>
@@ -13241,7 +13241,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="15" customHeight="1">
+    <row r="22" ht="16" customHeight="1">
       <c r="A22" s="16" t="inlineStr">
         <is>
           <t>STI-603</t>
@@ -13293,7 +13293,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1">
+    <row r="23" ht="16" customHeight="1">
       <c r="A23" s="17" t="inlineStr">
         <is>
           <t>STI-603</t>
@@ -13345,7 +13345,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="15" customHeight="1">
+    <row r="24" ht="16" customHeight="1">
       <c r="A24" s="20" t="inlineStr">
         <is>
           <t>Validasi Bobot</t>

</xml_diff>

<commit_message>
feat: finalize OBE 2026 curriculum documentation, tooling, and mapping analysis
</commit_message>
<xml_diff>
--- a/KURIKULUM2026_REVISI/011_IMPLEMENTASI_OBE_SISTEKIN2026_TABLES.xlsx
+++ b/KURIKULUM2026_REVISI/011_IMPLEMENTASI_OBE_SISTEKIN2026_TABLES.xlsx
@@ -751,14 +751,14 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="13" t="inlineStr">
         <is>
-          <t>SISTEKIN 2026 — Sheet 9: Template Evaluasi OBE - STI-601 (Integrasi AI)</t>
+          <t>SISTEKIN 2026 — Sheet 9: Template Evaluasi OBE - STI-624 (Integrasi AI)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>TEMPLATE EVALUASI OBE - STI-601 Integrasi Layanan Cerdas Berbasis AI</t>
+          <t>TEMPLATE EVALUASI OBE - STI-624 Integrasi Layanan Cerdas Berbasis AI</t>
         </is>
       </c>
     </row>
@@ -1093,14 +1093,14 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="13" t="inlineStr">
         <is>
-          <t>SISTEKIN 2026 — Sheet 10: Template Evaluasi OBE - STI-401 (Machine Learning)</t>
+          <t>SISTEKIN 2026 — Sheet 10: Template Evaluasi OBE - STI-413 (Machine Learning)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>TEMPLATE EVALUASI OBE - STI-401 Machine Learning (+P)</t>
+          <t>TEMPLATE EVALUASI OBE - STI-413 Machine Learning (+P)</t>
         </is>
       </c>
     </row>
@@ -1451,14 +1451,14 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="13" t="inlineStr">
         <is>
-          <t>SISTEKIN 2026 — Sheet 11: Template Evaluasi OBE - STI-303 (UI/UX)</t>
+          <t>SISTEKIN 2026 — Sheet 11: Template Evaluasi OBE - STI-308 (UI/UX)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>TEMPLATE EVALUASI OBE - STI-303 UI/UX Design &amp; Prototyping (+P)</t>
+          <t>TEMPLATE EVALUASI OBE - STI-308 UI/UX Design &amp; Prototyping (+P)</t>
         </is>
       </c>
     </row>
@@ -1792,14 +1792,14 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="13" t="inlineStr">
         <is>
-          <t>SISTEKIN 2026 — Sheet 12: Template Evaluasi OBE - STI-603 (Keamanan)</t>
+          <t>SISTEKIN 2026 — Sheet 12: Template Evaluasi OBE - STI-626 (Keamanan)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>TEMPLATE EVALUASI OBE - STI-603 Keamanan Informasi Lanjut</t>
+          <t>TEMPLATE EVALUASI OBE - STI-626 Keamanan Informasi Lanjut</t>
         </is>
       </c>
     </row>
@@ -2326,7 +2326,7 @@
       </c>
       <c r="D8" s="16" t="inlineStr">
         <is>
-          <t>STI-202 Aljabar Linear, FST-408 Statistika, FST-714 Skripsi</t>
+          <t>STI-205 Aljabar Linear, FST-408 Statistika, FST-714 Skripsi</t>
         </is>
       </c>
       <c r="E8" s="16" t="inlineStr">
@@ -2359,7 +2359,7 @@
       </c>
       <c r="D9" s="17" t="inlineStr">
         <is>
-          <t>STI-401 Machine Learning, STI-601 Integrasi AI, STI-503 Data Mining, FST-714 Skripsi</t>
+          <t>STI-413 Machine Learning, STI-624 Integrasi AI, STI-520 Data Mining, FST-714 Skripsi</t>
         </is>
       </c>
       <c r="E9" s="17" t="inlineStr">
@@ -2392,7 +2392,7 @@
       </c>
       <c r="D10" s="16" t="inlineStr">
         <is>
-          <t>STI-504 IoT, STI-602 Smart City, STI-603 Keamanan Lanjut, FST-714 Skripsi</t>
+          <t>STI-521 IoT, STI-625 Smart City, STI-626 Keamanan Lanjut, FST-714 Skripsi</t>
         </is>
       </c>
       <c r="E10" s="16" t="inlineStr">
@@ -2425,7 +2425,7 @@
       </c>
       <c r="D11" s="17" t="inlineStr">
         <is>
-          <t>STI-505 Mobile, STI-604 Platform Eng, FST-714 Skripsi</t>
+          <t>STI-522 Mobile, STI-627 Platform Eng, FST-714 Skripsi</t>
         </is>
       </c>
       <c r="E11" s="17" t="inlineStr">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="D12" s="16" t="inlineStr">
         <is>
-          <t>STI-501 Deep Learning, STI-601 Integrasi AI, FST-610 Capstone</t>
+          <t>STI-519 Deep Learning, STI-624 Integrasi AI, FST-610 Capstone</t>
         </is>
       </c>
       <c r="E12" s="16" t="inlineStr">
@@ -2491,7 +2491,7 @@
       </c>
       <c r="D13" s="17" t="inlineStr">
         <is>
-          <t>STI-501 Deep Learning, STI-503 Data Mining, STA-04 MLOps</t>
+          <t>STI-519 Deep Learning, STI-520 Data Mining, STA-04 MLOps</t>
         </is>
       </c>
       <c r="E13" s="17" t="inlineStr">
@@ -2524,7 +2524,7 @@
       </c>
       <c r="D14" s="16" t="inlineStr">
         <is>
-          <t>STI-504 IoT, STI-602 Smart City, STB-02 Cloud DevOps, FST-714 Skripsi</t>
+          <t>STI-521 IoT, STI-625 Smart City, STB-02 Cloud DevOps, FST-714 Skripsi</t>
         </is>
       </c>
       <c r="E14" s="16" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="D15" s="17" t="inlineStr">
         <is>
-          <t>STI-603 Keamanan Lanjut, STB-04 COBIT, FST-612 PKL</t>
+          <t>STI-626 Keamanan Lanjut, STB-04 COBIT, FST-612 PKL</t>
         </is>
       </c>
       <c r="E15" s="17" t="inlineStr">
@@ -2590,7 +2590,7 @@
       </c>
       <c r="D16" s="16" t="inlineStr">
         <is>
-          <t>STI-303 UI/UX, STI-505 Mobile, STI-604 Platform Eng, STC-01 UXR, FST-610 Capstone</t>
+          <t>STI-308 UI/UX, STI-522 Mobile, STI-627 Platform Eng, STC-01 UXR, FST-610 Capstone</t>
         </is>
       </c>
       <c r="E16" s="16" t="inlineStr">
@@ -2623,7 +2623,7 @@
       </c>
       <c r="D17" s="17" t="inlineStr">
         <is>
-          <t>STI-506 Manpro, STI-701 Startup, STC-06 Digital Product Mgmt</t>
+          <t>STI-523 Manpro, STI-728 Startup, STC-06 Digital Product Mgmt</t>
         </is>
       </c>
       <c r="E17" s="17" t="inlineStr">
@@ -3124,7 +3124,7 @@
       </c>
       <c r="B23" s="17" t="inlineStr">
         <is>
-          <t>STI-405 (Dasar Keamanan Informasi) = 2 SKS Teori (Sem 4). STI-602 (Smart City &amp; Pemerintahan Digital) = 2 SKS Teori Non-Praktikum (Sem 6).</t>
+          <t>STI-418 (Dasar Keamanan Informasi) = 2 SKS Teori (Sem 4). STI-625 (Smart City &amp; Pemerintahan Digital) = 2 SKS Teori Non-Praktikum (Sem 6).</t>
         </is>
       </c>
     </row>
@@ -6650,7 +6650,7 @@
       </c>
       <c r="B31" s="17" t="inlineStr">
         <is>
-          <t>STI-201</t>
+          <t>STI-204</t>
         </is>
       </c>
       <c r="C31" s="17" t="inlineStr">
@@ -6704,7 +6704,7 @@
       </c>
       <c r="B32" s="16" t="inlineStr">
         <is>
-          <t>STI-202</t>
+          <t>STI-205</t>
         </is>
       </c>
       <c r="C32" s="16" t="inlineStr">
@@ -6754,7 +6754,7 @@
       </c>
       <c r="B33" s="17" t="inlineStr">
         <is>
-          <t>STI-301</t>
+          <t>STI-306</t>
         </is>
       </c>
       <c r="C33" s="17" t="inlineStr">
@@ -6812,7 +6812,7 @@
       </c>
       <c r="B34" s="16" t="inlineStr">
         <is>
-          <t>STI-302</t>
+          <t>STI-307</t>
         </is>
       </c>
       <c r="C34" s="16" t="inlineStr">
@@ -6866,7 +6866,7 @@
       </c>
       <c r="B35" s="17" t="inlineStr">
         <is>
-          <t>STI-303</t>
+          <t>STI-308</t>
         </is>
       </c>
       <c r="C35" s="17" t="inlineStr">
@@ -6916,7 +6916,7 @@
       </c>
       <c r="B36" s="16" t="inlineStr">
         <is>
-          <t>STI-304</t>
+          <t>STI-309</t>
         </is>
       </c>
       <c r="C36" s="16" t="inlineStr">
@@ -6974,7 +6974,7 @@
       </c>
       <c r="B37" s="17" t="inlineStr">
         <is>
-          <t>STI-305</t>
+          <t>STI-310</t>
         </is>
       </c>
       <c r="C37" s="17" t="inlineStr">
@@ -7028,7 +7028,7 @@
       </c>
       <c r="B38" s="16" t="inlineStr">
         <is>
-          <t>STI-306</t>
+          <t>STI-311</t>
         </is>
       </c>
       <c r="C38" s="16" t="inlineStr">
@@ -7082,7 +7082,7 @@
       </c>
       <c r="B39" s="17" t="inlineStr">
         <is>
-          <t>STI-307</t>
+          <t>STI-312</t>
         </is>
       </c>
       <c r="C39" s="17" t="inlineStr">
@@ -7136,7 +7136,7 @@
       </c>
       <c r="B40" s="16" t="inlineStr">
         <is>
-          <t>STI-401</t>
+          <t>STI-413</t>
         </is>
       </c>
       <c r="C40" s="16" t="inlineStr">
@@ -7194,7 +7194,7 @@
       </c>
       <c r="B41" s="17" t="inlineStr">
         <is>
-          <t>STI-403</t>
+          <t>STI-414</t>
         </is>
       </c>
       <c r="C41" s="17" t="inlineStr">
@@ -7248,7 +7248,7 @@
       </c>
       <c r="B42" s="16" t="inlineStr">
         <is>
-          <t>STI-402</t>
+          <t>STI-415</t>
         </is>
       </c>
       <c r="C42" s="16" t="inlineStr">
@@ -7302,7 +7302,7 @@
       </c>
       <c r="B43" s="17" t="inlineStr">
         <is>
-          <t>STI-404</t>
+          <t>STI-417</t>
         </is>
       </c>
       <c r="C43" s="17" t="inlineStr">
@@ -7356,7 +7356,7 @@
       </c>
       <c r="B44" s="16" t="inlineStr">
         <is>
-          <t>STI-405</t>
+          <t>STI-418</t>
         </is>
       </c>
       <c r="C44" s="16" t="inlineStr">
@@ -7410,7 +7410,7 @@
       </c>
       <c r="B45" s="17" t="inlineStr">
         <is>
-          <t>STI-407</t>
+          <t>STI-416</t>
         </is>
       </c>
       <c r="C45" s="17" t="inlineStr">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="B46" s="16" t="inlineStr">
         <is>
-          <t>STI-501</t>
+          <t>STI-519</t>
         </is>
       </c>
       <c r="C46" s="16" t="inlineStr">
@@ -7518,7 +7518,7 @@
       </c>
       <c r="B47" s="17" t="inlineStr">
         <is>
-          <t>STI-503</t>
+          <t>STI-520</t>
         </is>
       </c>
       <c r="C47" s="17" t="inlineStr">
@@ -7572,7 +7572,7 @@
       </c>
       <c r="B48" s="16" t="inlineStr">
         <is>
-          <t>STI-504</t>
+          <t>STI-521</t>
         </is>
       </c>
       <c r="C48" s="16" t="inlineStr">
@@ -7626,7 +7626,7 @@
       </c>
       <c r="B49" s="17" t="inlineStr">
         <is>
-          <t>STI-505</t>
+          <t>STI-522</t>
         </is>
       </c>
       <c r="C49" s="17" t="inlineStr">
@@ -7680,7 +7680,7 @@
       </c>
       <c r="B50" s="16" t="inlineStr">
         <is>
-          <t>STI-506</t>
+          <t>STI-523</t>
         </is>
       </c>
       <c r="C50" s="16" t="inlineStr">
@@ -7730,7 +7730,7 @@
       </c>
       <c r="B51" s="17" t="inlineStr">
         <is>
-          <t>STI-601</t>
+          <t>STI-624</t>
         </is>
       </c>
       <c r="C51" s="17" t="inlineStr">
@@ -7784,7 +7784,7 @@
       </c>
       <c r="B52" s="16" t="inlineStr">
         <is>
-          <t>STI-602</t>
+          <t>STI-625</t>
         </is>
       </c>
       <c r="C52" s="16" t="inlineStr">
@@ -7838,7 +7838,7 @@
       </c>
       <c r="B53" s="17" t="inlineStr">
         <is>
-          <t>STI-603</t>
+          <t>STI-626</t>
         </is>
       </c>
       <c r="C53" s="17" t="inlineStr">
@@ -7896,7 +7896,7 @@
       </c>
       <c r="B54" s="16" t="inlineStr">
         <is>
-          <t>STI-604</t>
+          <t>STI-627</t>
         </is>
       </c>
       <c r="C54" s="16" t="inlineStr">
@@ -7950,7 +7950,7 @@
       </c>
       <c r="B55" s="17" t="inlineStr">
         <is>
-          <t>STI-701</t>
+          <t>STI-728</t>
         </is>
       </c>
       <c r="C55" s="17" t="inlineStr">
@@ -9235,7 +9235,7 @@
       </c>
       <c r="E5" s="17" t="inlineStr">
         <is>
-          <t>STI-201 Matematika Diskrit dan Logika (3) / STI-202 Aljabar Linear (3) / FST-203 Struktur Data &amp; Algoritma (3) / FST-204 Pengantar AI &amp; Data (2) / FST-205 Basic English (2) / FST-206 Etika &amp; Hukum Digital (2) / FST-207 Basis Data (3) / MKU-204 Kewirausahaan I (2)</t>
+          <t>STI-204 Matematika Diskrit dan Logika (3) / STI-205 Aljabar Linear (3) / FST-203 Struktur Data &amp; Algoritma (3) / FST-204 Pengantar AI &amp; Data (2) / FST-205 Basic English (2) / FST-206 Etika &amp; Hukum Digital (2) / FST-207 Basis Data (3) / MKU-204 Kewirausahaan I (2)</t>
         </is>
       </c>
       <c r="F5" s="19" t="inlineStr">
@@ -9272,7 +9272,7 @@
       </c>
       <c r="E6" s="16" t="inlineStr">
         <is>
-          <t>STI-301 APSI (3) / STI-302 Sistem Cerdas (2) / STI-303 UI/UX Design (3) / STI-304 RPL (3) / STI-305 Sistem Operasi (3) / STI-306 Web Front End (3) / STI-307 Jaringan Komputer (3)</t>
+          <t>STI-306 APSI (3) / STI-307 Sistem Cerdas (2) / STI-308 UI/UX Design (3) / STI-309 RPL (3) / STI-310 Sistem Operasi (3) / STI-311 Web Front End (3) / STI-312 Jaringan Komputer (3)</t>
         </is>
       </c>
       <c r="F6" s="18" t="inlineStr">
@@ -9309,7 +9309,7 @@
       </c>
       <c r="E7" s="17" t="inlineStr">
         <is>
-          <t>STI-401 Machine Learning (3) / STI-403 Pengantar NLP &amp; IR (2) / STI-402 DW &amp; BI (3) / STI-404 Cloud (3) / STI-405 Dasar Keamanan (2) / STI-407 Web Back End (3) / FST-408 Statistika (3) / MKU-405 KWN (2) / MKU-406 Agama II (0)</t>
+          <t>STI-413 Machine Learning (3) / STI-414 Pengantar NLP &amp; IR (2) / STI-415 DW &amp; BI (3) / STI-417 Cloud (3) / STI-418 Dasar Keamanan (2) / STI-416 Web Back End (3) / FST-408 Statistika (3) / MKU-405 KWN (2) / MKU-406 Agama II (0)</t>
         </is>
       </c>
       <c r="F7" s="19" t="inlineStr">
@@ -9319,7 +9319,7 @@
       </c>
       <c r="G7" s="19" t="inlineStr">
         <is>
-          <t>STI-405 = 2 SKS Teori. STI-403 = 2 SKS (+P). MKU-406 = 0 SKS kebijakan UWG</t>
+          <t>STI-418 = 2 SKS Teori. STI-414 = 2 SKS (+P). MKU-406 = 0 SKS kebijakan UWG</t>
         </is>
       </c>
     </row>
@@ -9346,7 +9346,7 @@
       </c>
       <c r="E8" s="16" t="inlineStr">
         <is>
-          <t>STI-501 Deep Learning (3) / STI-503 Data Mining (3) / STI-504 IoT (3) / STI-505 Mobile App (3) / STI-506 Manpro TI (3) / MKU-507 KPM (3) / MK Pilihan 1 (3) / MKU-508 KWU II (0)</t>
+          <t>STI-519 Deep Learning (3) / STI-520 Data Mining (3) / STI-521 IoT (3) / STI-522 Mobile App (3) / STI-523 Manpro TI (3) / MKU-507 KPM (3) / MK Pilihan 1 (3) / MKU-508 KWU II (0)</t>
         </is>
       </c>
       <c r="F8" s="18" t="inlineStr">
@@ -9383,7 +9383,7 @@
       </c>
       <c r="E9" s="17" t="inlineStr">
         <is>
-          <t>STI-601 Integrasi AI (3) / STI-602 Smart City (2) / STI-603 Keamanan Lanjut (3) / STI-604 Digital Platform Eng (3) / FST-611 Metopel (2) / MK Pilihan 2 (3) / MK Pilihan 3 (3)</t>
+          <t>STI-624 Integrasi AI (3) / STI-625 Smart City (2) / STI-626 Keamanan Lanjut (3) / STI-627 Digital Platform Eng (3) / FST-611 Metopel (2) / MK Pilihan 2 (3) / MK Pilihan 3 (3)</t>
         </is>
       </c>
       <c r="F9" s="19" t="inlineStr">
@@ -9393,7 +9393,7 @@
       </c>
       <c r="G9" s="19" t="inlineStr">
         <is>
-          <t>STI-602 = 2 SKS Teori Non-Praktikum. MBKM maks. 20 SKS</t>
+          <t>STI-625 = 2 SKS Teori Non-Praktikum. MBKM maks. 20 SKS</t>
         </is>
       </c>
     </row>
@@ -9420,7 +9420,7 @@
       </c>
       <c r="E10" s="16" t="inlineStr">
         <is>
-          <t>STI-701 Startup Digital (3) / FST-610 Capstone (3) / FST-612 PKL (3) / FST-613 Pra-Skripsi (2) / MK Pilihan 4 (3) / MK Pilihan 5 (3) / MK Pilihan 6 (3)</t>
+          <t>STI-728 Startup Digital (3) / FST-610 Capstone (3) / FST-612 PKL (3) / FST-613 Pra-Skripsi (2) / MK Pilihan 4 (3) / MK Pilihan 5 (3) / MK Pilihan 6 (3)</t>
         </is>
       </c>
       <c r="F10" s="18" t="inlineStr">
@@ -10075,7 +10075,7 @@
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="17" t="inlineStr">
         <is>
-          <t>STI-201</t>
+          <t>STI-204</t>
         </is>
       </c>
       <c r="B13" s="17" t="inlineStr">
@@ -10124,7 +10124,7 @@
     <row r="14" ht="16" customHeight="1">
       <c r="A14" s="16" t="inlineStr">
         <is>
-          <t>STI-202</t>
+          <t>STI-205</t>
         </is>
       </c>
       <c r="B14" s="16" t="inlineStr">
@@ -10406,7 +10406,7 @@
     <row r="20" ht="16" customHeight="1">
       <c r="A20" s="16" t="inlineStr">
         <is>
-          <t>STI-301</t>
+          <t>STI-306</t>
         </is>
       </c>
       <c r="B20" s="16" t="inlineStr">
@@ -10459,7 +10459,7 @@
     <row r="21" ht="16" customHeight="1">
       <c r="A21" s="17" t="inlineStr">
         <is>
-          <t>STI-302</t>
+          <t>STI-307</t>
         </is>
       </c>
       <c r="B21" s="17" t="inlineStr">
@@ -10508,7 +10508,7 @@
     <row r="22" ht="16" customHeight="1">
       <c r="A22" s="16" t="inlineStr">
         <is>
-          <t>STI-303</t>
+          <t>STI-308</t>
         </is>
       </c>
       <c r="B22" s="16" t="inlineStr">
@@ -10553,7 +10553,7 @@
     <row r="23" ht="16" customHeight="1">
       <c r="A23" s="17" t="inlineStr">
         <is>
-          <t>STI-304</t>
+          <t>STI-309</t>
         </is>
       </c>
       <c r="B23" s="17" t="inlineStr">
@@ -10606,7 +10606,7 @@
     <row r="24" ht="16" customHeight="1">
       <c r="A24" s="16" t="inlineStr">
         <is>
-          <t>STI-305</t>
+          <t>STI-310</t>
         </is>
       </c>
       <c r="B24" s="16" t="inlineStr">
@@ -10655,7 +10655,7 @@
     <row r="25" ht="16" customHeight="1">
       <c r="A25" s="17" t="inlineStr">
         <is>
-          <t>STI-306</t>
+          <t>STI-311</t>
         </is>
       </c>
       <c r="B25" s="17" t="inlineStr">
@@ -10704,7 +10704,7 @@
     <row r="26" ht="16" customHeight="1">
       <c r="A26" s="16" t="inlineStr">
         <is>
-          <t>STI-307</t>
+          <t>STI-312</t>
         </is>
       </c>
       <c r="B26" s="16" t="inlineStr">
@@ -10753,7 +10753,7 @@
     <row r="27" ht="16" customHeight="1">
       <c r="A27" s="17" t="inlineStr">
         <is>
-          <t>STI-401</t>
+          <t>STI-413</t>
         </is>
       </c>
       <c r="B27" s="17" t="inlineStr">
@@ -10806,7 +10806,7 @@
     <row r="28" ht="16" customHeight="1">
       <c r="A28" s="16" t="inlineStr">
         <is>
-          <t>STI-402</t>
+          <t>STI-415</t>
         </is>
       </c>
       <c r="B28" s="16" t="inlineStr">
@@ -10855,7 +10855,7 @@
     <row r="29" ht="16" customHeight="1">
       <c r="A29" s="17" t="inlineStr">
         <is>
-          <t>STI-404</t>
+          <t>STI-417</t>
         </is>
       </c>
       <c r="B29" s="17" t="inlineStr">
@@ -10904,7 +10904,7 @@
     <row r="30" ht="16" customHeight="1">
       <c r="A30" s="16" t="inlineStr">
         <is>
-          <t>STI-405</t>
+          <t>STI-418</t>
         </is>
       </c>
       <c r="B30" s="16" t="inlineStr">
@@ -10953,7 +10953,7 @@
     <row r="31" ht="16" customHeight="1">
       <c r="A31" s="17" t="inlineStr">
         <is>
-          <t>STI-407</t>
+          <t>STI-416</t>
         </is>
       </c>
       <c r="B31" s="17" t="inlineStr">
@@ -11051,7 +11051,7 @@
     <row r="33" ht="16" customHeight="1">
       <c r="A33" s="17" t="inlineStr">
         <is>
-          <t>STI-403</t>
+          <t>STI-414</t>
         </is>
       </c>
       <c r="B33" s="17" t="inlineStr">
@@ -11100,7 +11100,7 @@
     <row r="34" ht="16" customHeight="1">
       <c r="A34" s="16" t="inlineStr">
         <is>
-          <t>STI-501</t>
+          <t>STI-519</t>
         </is>
       </c>
       <c r="B34" s="16" t="inlineStr">
@@ -11149,7 +11149,7 @@
     <row r="35" ht="16" customHeight="1">
       <c r="A35" s="17" t="inlineStr">
         <is>
-          <t>STI-503</t>
+          <t>STI-520</t>
         </is>
       </c>
       <c r="B35" s="17" t="inlineStr">
@@ -11198,7 +11198,7 @@
     <row r="36" ht="16" customHeight="1">
       <c r="A36" s="16" t="inlineStr">
         <is>
-          <t>STI-504</t>
+          <t>STI-521</t>
         </is>
       </c>
       <c r="B36" s="16" t="inlineStr">
@@ -11247,7 +11247,7 @@
     <row r="37" ht="16" customHeight="1">
       <c r="A37" s="17" t="inlineStr">
         <is>
-          <t>STI-505</t>
+          <t>STI-522</t>
         </is>
       </c>
       <c r="B37" s="17" t="inlineStr">
@@ -11296,7 +11296,7 @@
     <row r="38" ht="16" customHeight="1">
       <c r="A38" s="16" t="inlineStr">
         <is>
-          <t>STI-506</t>
+          <t>STI-523</t>
         </is>
       </c>
       <c r="B38" s="16" t="inlineStr">
@@ -11390,7 +11390,7 @@
     <row r="40" ht="16" customHeight="1">
       <c r="A40" s="16" t="inlineStr">
         <is>
-          <t>STI-601</t>
+          <t>STI-624</t>
         </is>
       </c>
       <c r="B40" s="16" t="inlineStr">
@@ -11439,7 +11439,7 @@
     <row r="41" ht="16" customHeight="1">
       <c r="A41" s="17" t="inlineStr">
         <is>
-          <t>STI-602</t>
+          <t>STI-625</t>
         </is>
       </c>
       <c r="B41" s="17" t="inlineStr">
@@ -11488,7 +11488,7 @@
     <row r="42" ht="16" customHeight="1">
       <c r="A42" s="16" t="inlineStr">
         <is>
-          <t>STI-603</t>
+          <t>STI-626</t>
         </is>
       </c>
       <c r="B42" s="16" t="inlineStr">
@@ -11541,7 +11541,7 @@
     <row r="43" ht="16" customHeight="1">
       <c r="A43" s="17" t="inlineStr">
         <is>
-          <t>STI-604</t>
+          <t>STI-627</t>
         </is>
       </c>
       <c r="B43" s="17" t="inlineStr">
@@ -11643,7 +11643,7 @@
     <row r="45" ht="16" customHeight="1">
       <c r="A45" s="17" t="inlineStr">
         <is>
-          <t>STI-701</t>
+          <t>STI-728</t>
         </is>
       </c>
       <c r="B45" s="17" t="inlineStr">
@@ -12324,7 +12324,7 @@
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="16" t="inlineStr">
         <is>
-          <t>STI-601</t>
+          <t>STI-624</t>
         </is>
       </c>
       <c r="B4" s="16" t="inlineStr">
@@ -12376,7 +12376,7 @@
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="17" t="inlineStr">
         <is>
-          <t>STI-601</t>
+          <t>STI-624</t>
         </is>
       </c>
       <c r="B5" s="17" t="inlineStr">
@@ -12428,7 +12428,7 @@
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
-          <t>STI-601</t>
+          <t>STI-624</t>
         </is>
       </c>
       <c r="B6" s="16" t="inlineStr">
@@ -12480,7 +12480,7 @@
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
-          <t>STI-601</t>
+          <t>STI-624</t>
         </is>
       </c>
       <c r="B7" s="17" t="inlineStr">
@@ -12532,7 +12532,7 @@
     <row r="8" ht="16" customHeight="1">
       <c r="A8" s="16" t="inlineStr">
         <is>
-          <t>STI-401</t>
+          <t>STI-413</t>
         </is>
       </c>
       <c r="B8" s="16" t="inlineStr">
@@ -12584,7 +12584,7 @@
     <row r="9" ht="16" customHeight="1">
       <c r="A9" s="17" t="inlineStr">
         <is>
-          <t>STI-401</t>
+          <t>STI-413</t>
         </is>
       </c>
       <c r="B9" s="17" t="inlineStr">
@@ -12636,7 +12636,7 @@
     <row r="10" ht="16" customHeight="1">
       <c r="A10" s="16" t="inlineStr">
         <is>
-          <t>STI-401</t>
+          <t>STI-413</t>
         </is>
       </c>
       <c r="B10" s="16" t="inlineStr">
@@ -12688,7 +12688,7 @@
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="17" t="inlineStr">
         <is>
-          <t>STI-401</t>
+          <t>STI-413</t>
         </is>
       </c>
       <c r="B11" s="17" t="inlineStr">
@@ -12740,7 +12740,7 @@
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="16" t="inlineStr">
         <is>
-          <t>STI-504</t>
+          <t>STI-521</t>
         </is>
       </c>
       <c r="B12" s="16" t="inlineStr">
@@ -12792,7 +12792,7 @@
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="17" t="inlineStr">
         <is>
-          <t>STI-504</t>
+          <t>STI-521</t>
         </is>
       </c>
       <c r="B13" s="17" t="inlineStr">
@@ -12844,7 +12844,7 @@
     <row r="14" ht="16" customHeight="1">
       <c r="A14" s="16" t="inlineStr">
         <is>
-          <t>STI-504</t>
+          <t>STI-521</t>
         </is>
       </c>
       <c r="B14" s="16" t="inlineStr">
@@ -12896,7 +12896,7 @@
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="17" t="inlineStr">
         <is>
-          <t>STI-303</t>
+          <t>STI-308</t>
         </is>
       </c>
       <c r="B15" s="17" t="inlineStr">
@@ -12948,7 +12948,7 @@
     <row r="16" ht="16" customHeight="1">
       <c r="A16" s="16" t="inlineStr">
         <is>
-          <t>STI-303</t>
+          <t>STI-308</t>
         </is>
       </c>
       <c r="B16" s="16" t="inlineStr">
@@ -13000,7 +13000,7 @@
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="17" t="inlineStr">
         <is>
-          <t>STI-303</t>
+          <t>STI-308</t>
         </is>
       </c>
       <c r="B17" s="17" t="inlineStr">
@@ -13052,7 +13052,7 @@
     <row r="18" ht="16" customHeight="1">
       <c r="A18" s="16" t="inlineStr">
         <is>
-          <t>STI-604</t>
+          <t>STI-627</t>
         </is>
       </c>
       <c r="B18" s="16" t="inlineStr">
@@ -13104,7 +13104,7 @@
     <row r="19" ht="16" customHeight="1">
       <c r="A19" s="17" t="inlineStr">
         <is>
-          <t>STI-604</t>
+          <t>STI-627</t>
         </is>
       </c>
       <c r="B19" s="17" t="inlineStr">
@@ -13156,7 +13156,7 @@
     <row r="20" ht="16" customHeight="1">
       <c r="A20" s="16" t="inlineStr">
         <is>
-          <t>STI-604</t>
+          <t>STI-627</t>
         </is>
       </c>
       <c r="B20" s="16" t="inlineStr">
@@ -13208,7 +13208,7 @@
     <row r="21" ht="16" customHeight="1">
       <c r="A21" s="17" t="inlineStr">
         <is>
-          <t>STI-603</t>
+          <t>STI-626</t>
         </is>
       </c>
       <c r="B21" s="17" t="inlineStr">
@@ -13260,7 +13260,7 @@
     <row r="22" ht="16" customHeight="1">
       <c r="A22" s="16" t="inlineStr">
         <is>
-          <t>STI-603</t>
+          <t>STI-626</t>
         </is>
       </c>
       <c r="B22" s="16" t="inlineStr">
@@ -13312,7 +13312,7 @@
     <row r="23" ht="16" customHeight="1">
       <c r="A23" s="17" t="inlineStr">
         <is>
-          <t>STI-603</t>
+          <t>STI-626</t>
         </is>
       </c>
       <c r="B23" s="17" t="inlineStr">
@@ -13369,32 +13369,32 @@
       </c>
       <c r="B24" s="20" t="inlineStr">
         <is>
-          <t>STI-601: 100% OK</t>
+          <t>STI-624: 100% OK</t>
         </is>
       </c>
       <c r="C24" s="20" t="inlineStr">
         <is>
-          <t>STI-401: 100% OK</t>
+          <t>STI-413: 100% OK</t>
         </is>
       </c>
       <c r="D24" s="20" t="inlineStr">
         <is>
-          <t>STI-504: 100% OK</t>
+          <t>STI-521: 100% OK</t>
         </is>
       </c>
       <c r="E24" s="20" t="inlineStr">
         <is>
-          <t>STI-303: 100% OK</t>
+          <t>STI-308: 100% OK</t>
         </is>
       </c>
       <c r="F24" s="20" t="inlineStr">
         <is>
-          <t>STI-604: 100% OK</t>
+          <t>STI-627: 100% OK</t>
         </is>
       </c>
       <c r="G24" s="20" t="inlineStr">
         <is>
-          <t>STI-603: 100% OK</t>
+          <t>STI-626: 100% OK</t>
         </is>
       </c>
       <c r="H24" s="20" t="inlineStr"/>

</xml_diff>